<commit_message>
Adiciona campanha de doacao, acervo de arquivos e adaptacao a telas estreitas
</commit_message>
<xml_diff>
--- a/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
+++ b/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Divergências TCC1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos Funcionais'!$A$1:$H$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Divergências TCC1'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos Funcionais'!$A$1:$H$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Divergências TCC1'!$A$1:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H81,"CRÍTICA")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"CRÍTICA")</f>
         <v/>
       </c>
     </row>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H81,"ESSENCIAL")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"ESSENCIAL")</f>
         <v/>
       </c>
     </row>
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H81,"IMPORTANTE")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"IMPORTANTE")</f>
         <v/>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H81,"DESEJÁVEL")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"DESEJÁVEL")</f>
         <v/>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTA('Requisitos Funcionais'!B2:B81)</f>
+        <f>COUNTA('Requisitos Funcionais'!B2:B86)</f>
         <v/>
       </c>
     </row>
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3213,32 +3213,32 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>RF-PAI-001</t>
+          <t>RF-VOL-014</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Painel de quem conduz a turma</t>
+          <t>Publicar campanha de doação</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Painéis</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>Professor e monitor veem, num lugar só, as dúvidas sem resposta, os pedidos de ajuda abertos e os trabalhos em andamento das suas turmas.</t>
+          <t>A organização cadastra uma arrecadação de itens, como agasalhos ou alimentos, definindo como a contribuição será contada.</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>Composição das consultas dos módulos, restrita às disciplinas em que a pessoa leciona ou exerce monitoria. O monitor vê apenas onde é monitor.</t>
+          <t>Modalidade da oportunidade. A unidade é texto livre — peças de agasalho, quilos de alimento — porque qualquer lista fixa não teria a categoria da próxima campanha. Meta é opcional. Vagas e carga horária não se aplicam: campanha não limita participantes nem cumpre hora.</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
@@ -3253,32 +3253,32 @@
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>RF-PAI-002</t>
+          <t>RF-VOL-015</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Painel da organização parceira</t>
+          <t>Declarar doação</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Painéis</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>A organização vê suas oportunidades, quantos se inscreveram e quantos concluíram.</t>
+          <t>Estudante informa quanto pretende entregar à campanha.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Restrito às oportunidades da própria organização. A organização não participa do fórum: publica ações, acompanha inscrições e emite certificados.</t>
+          <t>POST em inscrever, com quantidade declarada e descrição opcional do item. É declaração de intenção: o valor fica registrado à parte e não entra na contagem da campanha até a organização confirmar o recebimento.</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H67" s="9" t="inlineStr">
@@ -3293,37 +3293,37 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-001</t>
+          <t>RF-VOL-016</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Entregar notificação em tempo real</t>
+          <t>Confirmar recebimento da doação</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>O aviso chega sem recarregar a página.</t>
+          <t>A organização registra quanto de fato recebeu, que pode divergir do que foi declarado.</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>WebSocket em /ws/notificacoes/ com Django Channels sobre Daphne. Sala por usuário. Camada em Redis quando disponível, com queda para camada em memória em implantação de instância única.</t>
+          <t>POST em concluir, com a quantidade confirmada. Sem valor informado, vale o declarado. O campo é somente leitura para o estudante: se ele pudesse registrar o próprio recebimento, o total da campanha deixaria de significar algo. Emite o certificado na mesma operação.</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -3333,27 +3333,27 @@
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-002</t>
+          <t>RF-VOL-017</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Listar notificações</t>
+          <t>Acompanhar a arrecadação</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê o histórico de avisos e quantos estão por ler.</t>
+          <t>A página da campanha mostra quanto já foi arrecadado e, havendo meta, o progresso em relação a ela.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>GET /api/notificacoes/ e /nao-lidas/.</t>
+          <t>Soma apenas as quantidades confirmadas em participações concluídas. Sem meta declarada não há barra de progresso: a barra precisa de um denominador, e inventar um faria a campanha parecer mais adiantada do que está.</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
@@ -3373,37 +3373,37 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-003</t>
+          <t>RF-VOL-018</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Marcar notificação como lida</t>
+          <t>Certificar participação em campanha</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>Usuário marca um aviso ou todos de uma vez.</t>
+          <t>Quem doou recebe certificado declarando a contribuição.</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>POST /api/notificacoes/{id}/marcar-lida/ e /marcar-todas-lidas/.</t>
+          <t>O texto do certificado muda com a modalidade: registra o que foi entregue e acrescenta que a organização atribui àquela participação o equivalente a um número de horas por ela definido. A formulação é deliberada — doar não é cumprir hora, e quem receber o documento precisa saber que avalia uma equivalência declarada pela entidade.</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3413,37 +3413,37 @@
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-004</t>
+          <t>RF-PAI-001</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Limpar notificações</t>
+          <t>Painel de quem conduz a turma</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Painéis</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Usuário descarta os avisos já lidos.</t>
+          <t>Professor e monitor veem, num lugar só, as dúvidas sem resposta, os pedidos de ajuda abertos e os trabalhos em andamento das suas turmas.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>POST /api/notificacoes/limpar/.</t>
+          <t>Composição das consultas dos módulos, restrita às disciplinas em que a pessoa leciona ou exerce monitoria. O monitor vê apenas onde é monitor.</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>DESEJÁVEL</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3453,37 +3453,37 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-005</t>
+          <t>RF-PAI-002</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Agrupar aviso por conversa</t>
+          <t>Painel da organização parceira</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Painéis</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>Uma conversa com muitas mensagens novas gera um aviso, e não um por mensagem.</t>
+          <t>A organização vê suas oportunidades, quantos se inscreveram e quantos concluíram.</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>Enquanto houver aviso não lido daquela conversa, não se cria outro. Sem isso, uma discussão ativa produziria dezenas de avisos e a pessoa desligaria todos.</t>
+          <t>Restrito às oportunidades da própria organização. A organização não participa do fórum: publica ações, acompanha inscrições e emite certificados.</t>
         </is>
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3493,32 +3493,32 @@
       </c>
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>RF-PRF-001</t>
+          <t>RF-NOT-001</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Visualizar perfil</t>
+          <t>Entregar notificação em tempo real</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Perfil</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê seus dados, foto, curso, período e disciplinas.</t>
+          <t>O aviso chega sem recarregar a página.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Compõe dados de /api/auth/me/ com o andamento por disciplina.</t>
+          <t>WebSocket em /ws/notificacoes/ com Django Channels sobre Daphne. Sala por usuário. Camada em Redis quando disponível, com queda para camada em memória em implantação de instância única.</t>
         </is>
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -3533,27 +3533,27 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>RF-PRF-002</t>
+          <t>RF-NOT-002</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Consultar histórico de participação</t>
+          <t>Listar notificações</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>Perfil</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>Usuário vê suas publicações, inscrições e certificados reunidos.</t>
+          <t>Usuário vê o histórico de avisos e quantos estão por ler.</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>Agrega as consultas de cada módulo na tela de perfil.</t>
+          <t>GET /api/notificacoes/ e /nao-lidas/.</t>
         </is>
       </c>
       <c r="G74" s="8" t="inlineStr">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3573,37 +3573,37 @@
       </c>
       <c r="B75" s="9" t="inlineStr">
         <is>
-          <t>RF-COO-001</t>
+          <t>RF-NOT-003</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Acompanhar o curso por disciplina</t>
+          <t>Marcar notificação como lida</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>A coordenação vê o movimento de cada disciplina do curso: volume de dúvidas, proporção respondida e tempo até a primeira resposta.</t>
+          <t>Usuário marca um aviso ou todos de uma vez.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Painel que agrega por disciplina e período. Identifica disciplina com muita dúvida sem resposta, que é o sinal que o painel existe para produzir.</t>
+          <t>POST /api/notificacoes/{id}/marcar-lida/ e /marcar-todas-lidas/.</t>
         </is>
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -3613,37 +3613,37 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>RF-COO-002</t>
+          <t>RF-NOT-004</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Detalhar uma disciplina</t>
+          <t>Limpar notificações</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>A coordenação abre uma disciplina e vê as dúvidas mais vistas e as sem resposta.</t>
+          <t>Usuário descarta os avisos já lidos.</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>Consulta por disciplina, ordenada pela razão entre visualizações e respostas.</t>
+          <t>POST /api/notificacoes/limpar/.</t>
         </is>
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -3653,32 +3653,32 @@
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>RF-COO-003</t>
+          <t>RF-NOT-005</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Importar a matriz curricular</t>
+          <t>Agrupar aviso por conversa</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>As disciplinas do curso entram na plataforma a partir do projeto pedagógico.</t>
+          <t>Uma conversa com muitas mensagens novas gera um aviso, e não um por mensagem.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Comando importar_matriz_ppc, que lê o ementário e cadastra código, nome, período e carga horária. A paridade do período define o semestre de oferta.</t>
+          <t>Enquanto houver aviso não lido daquela conversa, não se cria outro. Sem isso, uma discussão ativa produziria dezenas de avisos e a pessoa desligaria todos.</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H77" s="9" t="inlineStr">
@@ -3693,37 +3693,37 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>RF-AUD-001</t>
+          <t>RF-PRF-001</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Registrar ações sensíveis</t>
+          <t>Visualizar perfil</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Perfil</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>Ações de moderação e de gestão de vínculos ficam registradas.</t>
+          <t>Usuário vê seus dados, foto, curso, período e disciplinas.</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>Modelo de registro de auditoria, com autor, ação, alvo e momento. Consulta restrita à administração.</t>
+          <t>Compõe dados de /api/auth/me/ com o andamento por disciplina.</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3733,27 +3733,27 @@
       </c>
       <c r="B79" s="9" t="inlineStr">
         <is>
-          <t>RF-SIS-001</t>
+          <t>RF-PRF-002</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Alternar entre tema claro e escuro</t>
+          <t>Consultar histórico de participação</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Perfil</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Usuário escolhe o tema e a escolha permanece entre visitas.</t>
+          <t>Usuário vê suas publicações, inscrições e certificados reunidos.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Alternância por variáveis de cor no navegador, com a preferência guardada localmente. Todas as cores da interface vêm dessas variáveis: valor fixo escrito no código produz texto ilegível num dos dois temas.</t>
+          <t>Agrega as consultas de cada módulo na tela de perfil.</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
@@ -3773,37 +3773,37 @@
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>RF-SIS-002</t>
+          <t>RF-COO-001</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Consultar a documentação da API</t>
+          <t>Acompanhar o curso por disciplina</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Coordenação</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>A especificação da API fica acessível e navegável.</t>
+          <t>A coordenação vê o movimento de cada disciplina do curso: volume de dúvidas, proporção respondida e tempo até a primeira resposta.</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>Esquema OpenAPI gerado por drf-spectacular a partir das views e serializadores, com interface de navegação.</t>
+          <t>Painel que agrega por disciplina e período. Identifica disciplina com muita dúvida sem resposta, que é o sinal que o painel existe para produzir.</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Coordenação</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3813,42 +3813,242 @@
       </c>
       <c r="B81" s="9" t="inlineStr">
         <is>
+          <t>RF-COO-002</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>Detalhar uma disciplina</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>A coordenação abre uma disciplina e vê as dúvidas mais vistas e as sem resposta.</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>Consulta por disciplina, ordenada pela razão entre visualizações e respostas.</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>RF-COO-003</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Importar a matriz curricular</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>As disciplinas do curso entram na plataforma a partir do projeto pedagógico.</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Comando importar_matriz_ppc, que lê o ementário e cadastra código, nome, período e carga horária. A paridade do período define o semestre de oferta.</t>
+        </is>
+      </c>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
+        <is>
+          <t>RF-AUD-001</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>Registrar ações sensíveis</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="inlineStr">
+        <is>
+          <t>Ações de moderação e de gestão de vínculos ficam registradas.</t>
+        </is>
+      </c>
+      <c r="F83" s="9" t="inlineStr">
+        <is>
+          <t>Modelo de registro de auditoria, com autor, ação, alvo e momento. Consulta restrita à administração.</t>
+        </is>
+      </c>
+      <c r="G83" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="H83" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>RF-SIS-001</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Alternar entre tema claro e escuro</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>Usuário escolhe o tema e a escolha permanece entre visitas.</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>Alternância por variáveis de cor no navegador, com a preferência guardada localmente. Todas as cores da interface vêm dessas variáveis: valor fixo escrito no código produz texto ilegível num dos dois temas.</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
+          <t>RF-SIS-002</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>Consultar a documentação da API</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>A especificação da API fica acessível e navegável.</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>Esquema OpenAPI gerado por drf-spectacular a partir das views e serializadores, com interface de navegação.</t>
+        </is>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>Desenvolvedor</t>
+        </is>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
           <t>RF-SIS-003</t>
         </is>
       </c>
-      <c r="C81" s="9" t="inlineStr">
+      <c r="C86" s="8" t="inlineStr">
         <is>
           <t>Carregar dados de demonstração</t>
         </is>
       </c>
-      <c r="D81" s="9" t="inlineStr">
+      <c r="D86" s="8" t="inlineStr">
         <is>
           <t>Sistema</t>
         </is>
       </c>
-      <c r="E81" s="9" t="inlineStr">
+      <c r="E86" s="8" t="inlineStr">
         <is>
           <t>A plataforma pode ser povoada com um semestre completo para demonstração e avaliação.</t>
         </is>
       </c>
-      <c r="F81" s="9" t="inlineStr">
+      <c r="F86" s="8" t="inlineStr">
         <is>
           <t>Comando popular_demonstracao, com semente fixa para que a mesma execução produza sempre o mesmo conjunto. Gera disciplinas com ritmos distintos de atividade, deliberadamente incluindo uma sem professor atribuído, para que o painel de coordenação tenha o que apontar.</t>
         </is>
       </c>
-      <c r="G81" s="9" t="inlineStr">
+      <c r="G86" s="8" t="inlineStr">
         <is>
           <t>Coordenação</t>
         </is>
       </c>
-      <c r="H81" s="9" t="inlineStr">
+      <c r="H86" s="8" t="inlineStr">
         <is>
           <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H81"/>
+  <autoFilter ref="A1:H86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3859,7 +4059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4002,12 +4202,12 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Registro de doações e pontuação por item</t>
+          <t>Registro de doações</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Removido</t>
+          <t>Reformulado</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -4017,7 +4217,7 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Removido junto com o sistema de pontuação, pelo mesmo motivo.</t>
+          <t>O TCC1 previa doação como gerador de pontos, com fórmula progressiva por item. A pontuação foi removida, mas a doação em si retornou como modalidade própria de oportunidade: a organização publica uma campanha, define a unidade de contagem e uma meta opcional, e o estudante declara o que pretende entregar. O que mudou foi o propósito — antes o item valia pontos numa classificação, agora ele conta para uma arrecadação com destino concreto.</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4227,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Restrição de publicação por decisão pedagógica</t>
+          <t>Separação entre doação declarada e confirmada</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -4037,12 +4237,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>RF-FOR-015</t>
+          <t>Sem correspondência no TCC1</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Não estava previsto. Surgiu da distinção entre conteúdo que infringe regra, que é caso de denúncia, e resposta que entrega o exercício pronto, que não infringe nada e ainda assim prejudica a turma.</t>
+          <t>O desenho original registrava a doação num único valor. Na implementação ficou claro que intenção e recebimento são coisas distintas: somar o que os estudantes prometeram faria a campanha exibir uma arrecadação que nunca chegou. A confirmação passou a ser ato exclusivo da organização.</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4252,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Acervo de arquivos por disciplina</t>
+          <t>Restrição de publicação por decisão pedagógica</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -4062,12 +4262,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-014</t>
+          <t>RF-FOR-015</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Não estava previsto. Surgiu do uso: o material chegava por três caminhos diferentes e reencontrá-lo exigia lembrar por qual deles havia passado.</t>
+          <t>Não estava previsto. Surgiu da distinção entre conteúdo que infringe regra, que é caso de denúncia, e resposta que entrega o exercício pronto, que não infringe nada e ainda assim prejudica a turma.</t>
         </is>
       </c>
     </row>
@@ -4077,27 +4277,52 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
+          <t>Acervo de arquivos por disciplina</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Incorporado</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>RF-COL-014</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Não estava previsto. Surgiu do uso: o material chegava por três caminhos diferentes e reencontrá-lo exigia lembrar por qual deles havia passado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
           <t>Certificado com assinatura digital X.509</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Reduzido</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>RF-VOL-012 do TCC1</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>O certificado é emitido em PDF com código único de conferência. A assinatura criptográfica com certificado digital exigiria infraestrutura de chaves institucional, fora do alcance do trabalho.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:E10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(requisitos): atualiza RF e RNF e regenera as planilhas
- RF-FOR-012 (denunciar) passa a descrever a interface
- novo RF-FOR-023: sugerir dúvidas parecidas antes de publicar
- RNF-CON-004 atualizado para a suíte de 227 testes, ruff e tsc
- novo RNF-DES-008: busca interativa com debounce e cancelamento
Total: 86 requisitos funcionais e 51 não funcionais.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
+++ b/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Divergências TCC1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos Funcionais'!$A$1:$H$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos Funcionais'!$A$1:$H$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Divergências TCC1'!$A$1:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"CRÍTICA")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H87,"CRÍTICA")</f>
         <v/>
       </c>
     </row>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"ESSENCIAL")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H87,"ESSENCIAL")</f>
         <v/>
       </c>
     </row>
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"IMPORTANTE")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H87,"IMPORTANTE")</f>
         <v/>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H86,"DESEJÁVEL")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H87,"DESEJÁVEL")</f>
         <v/>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTA('Requisitos Funcionais'!B2:B86)</f>
+        <f>COUNTA('Requisitos Funcionais'!B2:B87)</f>
         <v/>
       </c>
     </row>
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>POST /api/forum/posts/{id}/denunciar/. Cria alerta com motivo e notifica quem modera a disciplina.</t>
+          <t>POST /api/forum/posts/{id}/denunciar/. Cria alerta com motivo e notifica quem modera a disciplina. Na interface, o botão Denunciar aparece no tópico e em cada resposta, abre um campo de motivo obrigatório e passa a indicar "Denúncia enviada" depois do envio. Não é oferecido ao autor do conteúdo, e a API recusa denúncia repetida enquanto a anterior estiver em análise.</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
@@ -1973,37 +1973,37 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-001</t>
+          <t>RF-FOR-023</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Propor trabalho em grupo</t>
+          <t>Sugerir dúvidas parecidas antes de publicar</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Colaboração</t>
+          <t>Fórum</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Professor cria um trabalho definindo quantidade de grupos, tamanho máximo, prazo e forma de montagem.</t>
+          <t>Ao escrever o título de uma nova dúvida, o aluno vê discussões semelhantes já existentes na disciplina e pode consultá-las antes de publicar.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/. Exige que a pessoa lecione a disciplina — a coordenação não passa nesta verificação, porque supervisionar não é participar da turma.</t>
+          <t>Tela de nova dúvida consulta GET /api/busca/ com a disciplina escolhida, até 5 resultados, 500 ms depois da última tecla e com título de ao menos 4 caracteres. Resultados repetidos do mesmo tópico são agrupados e os links abrem em outra aba, para não perder o texto digitado. Não é exibido a quem leciona, que publica avisos e material.</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Aluno/Monitor</t>
         </is>
       </c>
       <c r="H35" s="9" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2013,12 +2013,12 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-002</t>
+          <t>RF-COL-001</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Anexar material ao enunciado</t>
+          <t>Propor trabalho em grupo</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -2028,12 +2028,12 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Professor anexa a especificação, a base de dados e o esqueleto de código ao próprio trabalho.</t>
+          <t>Professor cria um trabalho definindo quantidade de grupos, tamanho máximo, prazo e forma de montagem.</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/{id}/anexar/ e remoção correspondente. Lista de tipos aceitos e limite de tamanho no servidor. Fica no trabalho, e não no grupo: é material da turma inteira. Sem este espaço, o professor distribuiria por outro canal e o enunciado ficaria separado dos arquivos.</t>
+          <t>POST /api/colaboracao/trabalhos/. Exige que a pessoa lecione a disciplina — a coordenação não passa nesta verificação, porque supervisionar não é participar da turma.</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -2053,12 +2053,12 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-003</t>
+          <t>RF-COL-002</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Criar grupos vazios</t>
+          <t>Anexar material ao enunciado</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
@@ -2068,12 +2068,12 @@
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Sistema gera os grupos previstos para que os alunos escolham onde entrar.</t>
+          <t>Professor anexa a especificação, a base de dados e o esqueleto de código ao próprio trabalho.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/{id}/criar-grupos/. Cria a conversa privada de cada grupo junto.</t>
+          <t>POST /api/colaboracao/trabalhos/{id}/anexar/ e remoção correspondente. Lista de tipos aceitos e limite de tamanho no servidor. Fica no trabalho, e não no grupo: é material da turma inteira. Sem este espaço, o professor distribuiria por outro canal e o enunciado ficaria separado dos arquivos.</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
@@ -2093,12 +2093,12 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-004</t>
+          <t>RF-COL-003</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Sortear a composição dos grupos</t>
+          <t>Criar grupos vazios</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
@@ -2108,12 +2108,12 @@
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Distribuição aleatória dos matriculados entre os grupos.</t>
+          <t>Sistema gera os grupos previstos para que os alunos escolham onde entrar.</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/{id}/sortear/. Respeita o tamanho máximo e sincroniza os participantes das conversas.</t>
+          <t>POST /api/colaboracao/trabalhos/{id}/criar-grupos/. Cria a conversa privada de cada grupo junto.</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2133,12 +2133,12 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-005</t>
+          <t>RF-COL-004</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Entrar em grupo</t>
+          <t>Sortear a composição dos grupos</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -2148,22 +2148,22 @@
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Aluno escolhe o grupo de que quer participar.</t>
+          <t>Distribuição aleatória dos matriculados entre os grupos.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/grupos/{id}/entrar/. Recusa se o grupo estiver cheio ou se a pessoa já estiver em outro grupo do mesmo trabalho. Insere na conversa do grupo.</t>
+          <t>POST /api/colaboracao/trabalhos/{id}/sortear/. Respeita o tamanho máximo e sincroniza os participantes das conversas.</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H39" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2173,12 +2173,12 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-006</t>
+          <t>RF-COL-005</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Sair de grupo</t>
+          <t>Entrar em grupo</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -2188,12 +2188,12 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Aluno deixa o grupo, com confirmação antes.</t>
+          <t>Aluno escolhe o grupo de que quer participar.</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/grupos/{id}/sair/. Remove da conversa e atualiza a contagem de participantes.</t>
+          <t>POST /api/colaboracao/grupos/{id}/entrar/. Recusa se o grupo estiver cheio ou se a pessoa já estiver em outro grupo do mesmo trabalho. Insere na conversa do grupo.</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2213,12 +2213,12 @@
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-007</t>
+          <t>RF-COL-006</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Definir responsável pelo grupo</t>
+          <t>Sair de grupo</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -2228,22 +2228,22 @@
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>O grupo indica quem responde por ele.</t>
+          <t>Aluno deixa o grupo, com confirmação antes.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/grupos/{id}/definir-lider/.</t>
+          <t>POST /api/colaboracao/grupos/{id}/sair/. Remove da conversa e atualiza a contagem de participantes.</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>Aluno/Professor</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>DESEJÁVEL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2253,12 +2253,12 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-008</t>
+          <t>RF-COL-007</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Conversar em tempo real no grupo</t>
+          <t>Definir responsável pelo grupo</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -2268,22 +2268,22 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Os integrantes trocam mensagens, imagens, documentos e áudio no espaço privado do grupo.</t>
+          <t>O grupo indica quem responde por ele.</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>GET e POST /api/colaboracao/conversas/{id}/mensagens/, com entrega imediata por WebSocket via Django Channels. A conversa é privada aos integrantes, inclusive em relação ao professor. É a decisão que sustenta o módulo: sem privacidade, os grupos migram para aplicativos externos e o material se perde no fim do semestre.</t>
+          <t>POST /api/colaboracao/grupos/{id}/definir-lider/.</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Aluno/Professor</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -2293,12 +2293,12 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-009</t>
+          <t>RF-COL-008</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Excluir mensagem enviada</t>
+          <t>Conversar em tempo real no grupo</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
@@ -2308,22 +2308,22 @@
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Autor apaga uma mensagem dentro de um prazo curto após o envio.</t>
+          <t>Os integrantes trocam mensagens, imagens, documentos e áudio no espaço privado do grupo.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>DELETE /api/colaboracao/mensagens/{id}/. Janela de três minutos, verificação de autoria e exclusão lógica. Recusa se a mensagem já tiver originado um pedido de ajuda, para não apagar o que já foi encaminhado a terceiros. Anuncia a exclusão aos demais pelo WebSocket.</t>
+          <t>GET e POST /api/colaboracao/conversas/{id}/mensagens/, com entrega imediata por WebSocket via Django Channels. A conversa é privada aos integrantes, inclusive em relação ao professor. É a decisão que sustenta o módulo: sem privacidade, os grupos migram para aplicativos externos e o material se perde no fim do semestre.</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>Autor</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -2333,12 +2333,12 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-010</t>
+          <t>RF-COL-009</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Registrar leitura da conversa</t>
+          <t>Excluir mensagem enviada</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -2348,17 +2348,17 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>O contador de mensagens não lidas zera quando a pessoa abre a conversa.</t>
+          <t>Autor apaga uma mensagem dentro de um prazo curto após o envio.</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/conversas/{id}/marcar-lida/. O marcador fica no participante, e não na mensagem: guardar um registro por mensagem e por pessoa inviabilizaria qualquer conversa ativa.</t>
+          <t>DELETE /api/colaboracao/mensagens/{id}/. Janela de três minutos, verificação de autoria e exclusão lógica. Recusa se a mensagem já tiver originado um pedido de ajuda, para não apagar o que já foi encaminhado a terceiros. Anuncia a exclusão aos demais pelo WebSocket.</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Autor</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr">
@@ -2373,12 +2373,12 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-011</t>
+          <t>RF-COL-010</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Encaminhar dúvida do grupo</t>
+          <t>Registrar leitura da conversa</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
@@ -2388,12 +2388,12 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>O grupo marca uma mensagem e a encaminha a quem conduz a turma, com uma descrição do problema.</t>
+          <t>O contador de mensagens não lidas zera quando a pessoa abre a conversa.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/conversas/{id}/pedir-ajuda/. O destino é decidido pelo sistema: monitoria quando a disciplina tem monitor, professor quando não tem. Só a mensagem marcada e a descrição atravessam — a conversa em volta continua invisível.</t>
+          <t>POST /api/colaboracao/conversas/{id}/marcar-lida/. O marcador fica no participante, e não na mensagem: guardar um registro por mensagem e por pessoa inviabilizaria qualquer conversa ativa.</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="H45" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2413,12 +2413,12 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-012</t>
+          <t>RF-COL-011</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Assumir pedido de ajuda</t>
+          <t>Encaminhar dúvida do grupo</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
@@ -2428,22 +2428,22 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>Monitor ou professor assume o atendimento.</t>
+          <t>O grupo marca uma mensagem e a encaminha a quem conduz a turma, com uma descrição do problema.</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/ajuda/{id}/assumir/. Evita que dois atendam o mesmo pedido.</t>
+          <t>POST /api/colaboracao/conversas/{id}/pedir-ajuda/. O destino é decidido pelo sistema: monitoria quando a disciplina tem monitor, professor quando não tem. Só a mensagem marcada e a descrição atravessam — a conversa em volta continua invisível.</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Monitor/Professor</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2453,12 +2453,12 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-013</t>
+          <t>RF-COL-012</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Responder pedido de ajuda</t>
+          <t>Assumir pedido de ajuda</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
@@ -2468,12 +2468,12 @@
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Quem assumiu responde e a resposta chega ao grupo.</t>
+          <t>Monitor ou professor assume o atendimento.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/ajuda/{id}/responder/. Registra a resposta e notifica os integrantes.</t>
+          <t>POST /api/colaboracao/ajuda/{id}/assumir/. Evita que dois atendam o mesmo pedido.</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="H47" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2493,12 +2493,12 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-014</t>
+          <t>RF-COL-013</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Reunir arquivos por disciplina</t>
+          <t>Responder pedido de ajuda</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
@@ -2508,22 +2508,22 @@
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>Usuário encontra num lugar só todo o material que passou por ele, separado por matéria.</t>
+          <t>Quem assumiu responde e a resposta chega ao grupo.</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/arquivos/. Reúne três origens: anexo de conversa, material de trabalho e anexo de publicação. Sem modelo novo e sem cópia: a consulta lê o que já está gravado, mantendo o recorte de permissão de cada origem. Anexo de conversa só aparece para quem participa dela.</t>
+          <t>POST /api/colaboracao/ajuda/{id}/responder/. Registra a resposta e notifica os integrantes.</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>Aluno/Monitor/Professor</t>
+          <t>Monitor/Professor</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2533,12 +2533,12 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-015</t>
+          <t>RF-COL-014</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Consultar trabalhos da disciplina</t>
+          <t>Reunir arquivos por disciplina</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
@@ -2548,12 +2548,12 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê os trabalhos propostos, o prazo e a situação do próprio grupo.</t>
+          <t>Usuário encontra num lugar só todo o material que passou por ele, separado por matéria.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/trabalhos/. Filtra pelas disciplinas de vínculo. Quem não tem vínculo com nenhuma disciplina não alcança esta tela: a aba sequer aparece, porque toda ação disponível ali terminaria em erro.</t>
+          <t>GET /api/colaboracao/arquivos/. Reúne três origens: anexo de conversa, material de trabalho e anexo de publicação. Sem modelo novo e sem cópia: a consulta lê o que já está gravado, mantendo o recorte de permissão de cada origem. Anexo de conversa só aparece para quem participa dela.</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2573,12 +2573,12 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-016</t>
+          <t>RF-COL-015</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Consultar composição dos grupos</t>
+          <t>Consultar trabalhos da disciplina</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -2588,17 +2588,17 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>Quem conduz a turma vê como os grupos ficaram formados.</t>
+          <t>Usuário vê os trabalhos propostos, o prazo e a situação do próprio grupo.</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/grupos/. O professor enxerga a composição e o andamento, mas não entra na conversa privada da equipe.</t>
+          <t>GET /api/colaboracao/trabalhos/. Filtra pelas disciplinas de vínculo. Quem não tem vínculo com nenhuma disciplina não alcança esta tela: a aba sequer aparece, porque toda ação disponível ali terminaria em erro.</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Aluno/Monitor/Professor</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
@@ -2613,12 +2613,12 @@
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-017</t>
+          <t>RF-COL-016</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Listar conversas com pendências</t>
+          <t>Consultar composição dos grupos</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
@@ -2628,17 +2628,17 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê suas conversas com a quantidade de mensagens por ler.</t>
+          <t>Quem conduz a turma vê como os grupos ficaram formados.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/conversas/. Filtra por participação e calcula as não lidas a partir do marcador de leitura de cada participante.</t>
+          <t>GET /api/colaboracao/grupos/. O professor enxerga a composição e o andamento, mas não entra na conversa privada da equipe.</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>Aluno/Monitor/Professor</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H51" s="9" t="inlineStr">
@@ -2653,12 +2653,12 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-018</t>
+          <t>RF-COL-017</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Acompanhar a fila de pedidos de ajuda</t>
+          <t>Listar conversas com pendências</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -2668,17 +2668,17 @@
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>Quem conduz a turma vê os pedidos abertos, em atendimento e resolvidos.</t>
+          <t>Usuário vê suas conversas com a quantidade de mensagens por ler.</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/ajuda/. O destino do pedido decide quem o enxerga: monitoria quando a disciplina tem monitor, professor quando não tem.</t>
+          <t>GET /api/colaboracao/conversas/. Filtra por participação e calcula as não lidas a partir do marcador de leitura de cada participante.</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>Monitor/Professor</t>
+          <t>Aluno/Monitor/Professor</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
@@ -2693,32 +2693,32 @@
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-001</t>
+          <t>RF-COL-018</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Publicar oportunidade</t>
+          <t>Acompanhar a fila de pedidos de ajuda</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Voluntariado</t>
+          <t>Colaboração</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Organização parceira cadastra uma ação de voluntariado com período, vagas, carga horária e local.</t>
+          <t>Quem conduz a turma vê os pedidos abertos, em atendimento e resolvidos.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/oportunidades/. Restrito ao perfil de organização.</t>
+          <t>GET /api/colaboracao/ajuda/. O destino do pedido decide quem o enxerga: monitoria quando a disciplina tem monitor, professor quando não tem.</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Monitor/Professor</t>
         </is>
       </c>
       <c r="H53" s="9" t="inlineStr">
@@ -2733,12 +2733,12 @@
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-002</t>
+          <t>RF-VOL-001</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Consultar oportunidades</t>
+          <t>Publicar oportunidade</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
@@ -2748,17 +2748,17 @@
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>Estudante vê as ações disponíveis, com filtro por situação e busca por texto.</t>
+          <t>Organização parceira cadastra uma ação de voluntariado com período, vagas, carga horária e local.</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>GET /api/voluntariado/oportunidades/. Informa vagas preenchidas e total.</t>
+          <t>POST /api/voluntariado/oportunidades/. Restrito ao perfil de organização.</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
@@ -2773,12 +2773,12 @@
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-003</t>
+          <t>RF-VOL-002</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Inscrever-se em oportunidade</t>
+          <t>Consultar oportunidades</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -2788,12 +2788,12 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Estudante se candidata a uma vaga.</t>
+          <t>Estudante vê as ações disponíveis, com filtro por situação e busca por texto.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/oportunidades/{id}/inscrever/. Unicidade por par pessoa e oportunidade. Verifica vaga disponível dentro de transação, para que duas inscrições simultâneas não ultrapassem o limite.</t>
+          <t>GET /api/voluntariado/oportunidades/. Informa vagas preenchidas e total.</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
@@ -2813,12 +2813,12 @@
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-004</t>
+          <t>RF-VOL-003</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Desistir da inscrição</t>
+          <t>Inscrever-se em oportunidade</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
@@ -2828,12 +2828,12 @@
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>Estudante cancela a própria inscrição e libera a vaga.</t>
+          <t>Estudante se candidata a uma vaga.</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/inscricoes/{id}/desistir/.</t>
+          <t>POST /api/voluntariado/oportunidades/{id}/inscrever/. Unicidade por par pessoa e oportunidade. Verifica vaga disponível dentro de transação, para que duas inscrições simultâneas não ultrapassem o limite.</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2853,12 +2853,12 @@
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-005</t>
+          <t>RF-VOL-004</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Aprovar ou rejeitar inscrição</t>
+          <t>Desistir da inscrição</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -2868,22 +2868,22 @@
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>A organização decide quem participa.</t>
+          <t>Estudante cancela a própria inscrição e libera a vaga.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/inscricoes/{id}/aprovar/ e rejeitar. Notifica o candidato da decisão.</t>
+          <t>POST /api/voluntariado/inscricoes/{id}/desistir/.</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H57" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2893,12 +2893,12 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-006</t>
+          <t>RF-VOL-005</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Remover participante</t>
+          <t>Aprovar ou rejeitar inscrição</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -2908,12 +2908,12 @@
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>A organização retira alguém já aprovado.</t>
+          <t>A organização decide quem participa.</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/inscricoes/{id}/remover/. Devolve a vaga.</t>
+          <t>POST /api/voluntariado/inscricoes/{id}/aprovar/ e rejeitar. Notifica o candidato da decisão.</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2933,12 +2933,12 @@
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-007</t>
+          <t>RF-VOL-006</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Concluir participação</t>
+          <t>Remover participante</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
@@ -2948,12 +2948,12 @@
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>A organização confirma que a pessoa cumpriu a ação, o que dispara a emissão do certificado.</t>
+          <t>A organização retira alguém já aprovado.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/inscricoes/{id}/concluir/. Registra a conclusão e gera o certificado na sequência.</t>
+          <t>POST /api/voluntariado/inscricoes/{id}/remover/. Devolve a vaga.</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2973,12 +2973,12 @@
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-008</t>
+          <t>RF-VOL-007</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Emitir certificado em PDF</t>
+          <t>Concluir participação</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
@@ -2988,17 +2988,17 @@
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t>Certificado de participação com código de verificação, para aproveitamento das horas como atividade complementar.</t>
+          <t>A organização confirma que a pessoa cumpriu a ação, o que dispara a emissão do certificado.</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>Geração com WeasyPrint a partir de modelo HTML, com identidade visual da UNIFEI, dados da ação, carga horária e código único de conferência.</t>
+          <t>POST /api/voluntariado/inscricoes/{id}/concluir/. Registra a conclusão e gera o certificado na sequência.</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
@@ -3013,12 +3013,12 @@
       </c>
       <c r="B61" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-009</t>
+          <t>RF-VOL-008</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Consultar certificados</t>
+          <t>Emitir certificado em PDF</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
@@ -3028,22 +3028,22 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Estudante acessa e baixa os certificados que recebeu.</t>
+          <t>Certificado de participação com código de verificação, para aproveitamento das horas como atividade complementar.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>GET /api/voluntariado/certificados/.</t>
+          <t>Geração com WeasyPrint a partir de modelo HTML, com identidade visual da UNIFEI, dados da ação, carga horária e código único de conferência.</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -3053,12 +3053,12 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-010</t>
+          <t>RF-VOL-009</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Acompanhar inscritos</t>
+          <t>Consultar certificados</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
@@ -3068,17 +3068,17 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>A organização vê quem se inscreveu e em que situação está cada inscrição.</t>
+          <t>Estudante acessa e baixa os certificados que recebeu.</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>GET /api/voluntariado/oportunidades/{id}/inscricoes/.</t>
+          <t>GET /api/voluntariado/certificados/.</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
@@ -3093,12 +3093,12 @@
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-011</t>
+          <t>RF-VOL-010</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Editar oportunidade publicada</t>
+          <t>Acompanhar inscritos</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -3108,12 +3108,12 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>A organização corrige dados da ação já publicada.</t>
+          <t>A organização vê quem se inscreveu e em que situação está cada inscrição.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>PUT /api/voluntariado/oportunidades/{id}/. Verifica que a organização é a autora. Alteração de data notifica os inscritos.</t>
+          <t>GET /api/voluntariado/oportunidades/{id}/inscricoes/.</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="H63" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3133,12 +3133,12 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-012</t>
+          <t>RF-VOL-011</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>Encerrar oportunidade</t>
+          <t>Editar oportunidade publicada</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
@@ -3148,12 +3148,12 @@
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>A organização encerra as inscrições sem apagar o registro.</t>
+          <t>A organização corrige dados da ação já publicada.</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>Alteração de situação, e não remoção. Quem participou precisa de um caminho de volta até a ação para alcançar o certificado.</t>
+          <t>PUT /api/voluntariado/oportunidades/{id}/. Verifica que a organização é a autora. Alteração de data notifica os inscritos.</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
@@ -3163,7 +3163,7 @@
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -3173,12 +3173,12 @@
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-013</t>
+          <t>RF-VOL-012</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Consultar as próprias inscrições</t>
+          <t>Encerrar oportunidade</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -3188,17 +3188,17 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Estudante acompanha em que situação está cada candidatura.</t>
+          <t>A organização encerra as inscrições sem apagar o registro.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>GET /api/voluntariado/inscricoes/minhas/.</t>
+          <t>Alteração de situação, e não remoção. Quem participou precisa de um caminho de volta até a ação para alcançar o certificado.</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H65" s="9" t="inlineStr">
@@ -3213,12 +3213,12 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-014</t>
+          <t>RF-VOL-013</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Publicar campanha de doação</t>
+          <t>Consultar as próprias inscrições</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
@@ -3228,17 +3228,17 @@
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>A organização cadastra uma arrecadação de itens, como agasalhos ou alimentos, definindo como a contribuição será contada.</t>
+          <t>Estudante acompanha em que situação está cada candidatura.</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>Modalidade da oportunidade. A unidade é texto livre — peças de agasalho, quilos de alimento — porque qualquer lista fixa não teria a categoria da próxima campanha. Meta é opcional. Vagas e carga horária não se aplicam: campanha não limita participantes nem cumpre hora.</t>
+          <t>GET /api/voluntariado/inscricoes/minhas/.</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
@@ -3253,12 +3253,12 @@
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-015</t>
+          <t>RF-VOL-014</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Declarar doação</t>
+          <t>Publicar campanha de doação</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -3268,17 +3268,17 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Estudante informa quanto pretende entregar à campanha.</t>
+          <t>A organização cadastra uma arrecadação de itens, como agasalhos ou alimentos, definindo como a contribuição será contada.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>POST em inscrever, com quantidade declarada e descrição opcional do item. É declaração de intenção: o valor fica registrado à parte e não entra na contagem da campanha até a organização confirmar o recebimento.</t>
+          <t>Modalidade da oportunidade. A unidade é texto livre — peças de agasalho, quilos de alimento — porque qualquer lista fixa não teria a categoria da próxima campanha. Meta é opcional. Vagas e carga horária não se aplicam: campanha não limita participantes nem cumpre hora.</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H67" s="9" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-016</t>
+          <t>RF-VOL-015</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Confirmar recebimento da doação</t>
+          <t>Declarar doação</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
@@ -3308,22 +3308,22 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>A organização registra quanto de fato recebeu, que pode divergir do que foi declarado.</t>
+          <t>Estudante informa quanto pretende entregar à campanha.</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>POST em concluir, com a quantidade confirmada. Sem valor informado, vale o declarado. O campo é somente leitura para o estudante: se ele pudesse registrar o próprio recebimento, o total da campanha deixaria de significar algo. Emite o certificado na mesma operação.</t>
+          <t>POST em inscrever, com quantidade declarada e descrição opcional do item. É declaração de intenção: o valor fica registrado à parte e não entra na contagem da campanha até a organização confirmar o recebimento.</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3333,12 +3333,12 @@
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-017</t>
+          <t>RF-VOL-016</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Acompanhar a arrecadação</t>
+          <t>Confirmar recebimento da doação</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -3348,22 +3348,22 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>A página da campanha mostra quanto já foi arrecadado e, havendo meta, o progresso em relação a ela.</t>
+          <t>A organização registra quanto de fato recebeu, que pode divergir do que foi declarado.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Soma apenas as quantidades confirmadas em participações concluídas. Sem meta declarada não há barra de progresso: a barra precisa de um denominador, e inventar um faria a campanha parecer mais adiantada do que está.</t>
+          <t>POST em concluir, com a quantidade confirmada. Sem valor informado, vale o declarado. O campo é somente leitura para o estudante: se ele pudesse registrar o próprio recebimento, o total da campanha deixaria de significar algo. Emite o certificado na mesma operação.</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H69" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -3373,12 +3373,12 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-018</t>
+          <t>RF-VOL-017</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Certificar participação em campanha</t>
+          <t>Acompanhar a arrecadação</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
@@ -3388,17 +3388,17 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>Quem doou recebe certificado declarando a contribuição.</t>
+          <t>A página da campanha mostra quanto já foi arrecadado e, havendo meta, o progresso em relação a ela.</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>O texto do certificado muda com a modalidade: registra o que foi entregue e acrescenta que a organização atribui àquela participação o equivalente a um número de horas por ela definido. A formulação é deliberada — doar não é cumprir hora, e quem receber o documento precisa saber que avalia uma equivalência declarada pela entidade.</t>
+          <t>Soma apenas as quantidades confirmadas em participações concluídas. Sem meta declarada não há barra de progresso: a barra precisa de um denominador, e inventar um faria a campanha parecer mais adiantada do que está.</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
@@ -3413,32 +3413,32 @@
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>RF-PAI-001</t>
+          <t>RF-VOL-018</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Painel de quem conduz a turma</t>
+          <t>Certificar participação em campanha</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Painéis</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Professor e monitor veem, num lugar só, as dúvidas sem resposta, os pedidos de ajuda abertos e os trabalhos em andamento das suas turmas.</t>
+          <t>Quem doou recebe certificado declarando a contribuição.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Composição das consultas dos módulos, restrita às disciplinas em que a pessoa leciona ou exerce monitoria. O monitor vê apenas onde é monitor.</t>
+          <t>O texto do certificado muda com a modalidade: registra o que foi entregue e acrescenta que a organização atribui àquela participação o equivalente a um número de horas por ela definido. A formulação é deliberada — doar não é cumprir hora, e quem receber o documento precisa saber que avalia uma equivalência declarada pela entidade.</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H71" s="9" t="inlineStr">
@@ -3453,12 +3453,12 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>RF-PAI-002</t>
+          <t>RF-PAI-001</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Painel da organização parceira</t>
+          <t>Painel de quem conduz a turma</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
@@ -3468,17 +3468,17 @@
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>A organização vê suas oportunidades, quantos se inscreveram e quantos concluíram.</t>
+          <t>Professor e monitor veem, num lugar só, as dúvidas sem resposta, os pedidos de ajuda abertos e os trabalhos em andamento das suas turmas.</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>Restrito às oportunidades da própria organização. A organização não participa do fórum: publica ações, acompanha inscrições e emite certificados.</t>
+          <t>Composição das consultas dos módulos, restrita às disciplinas em que a pessoa leciona ou exerce monitoria. O monitor vê apenas onde é monitor.</t>
         </is>
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -3493,32 +3493,32 @@
       </c>
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-001</t>
+          <t>RF-PAI-002</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Entregar notificação em tempo real</t>
+          <t>Painel da organização parceira</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Painéis</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>O aviso chega sem recarregar a página.</t>
+          <t>A organização vê suas oportunidades, quantos se inscreveram e quantos concluíram.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>WebSocket em /ws/notificacoes/ com Django Channels sobre Daphne. Sala por usuário. Camada em Redis quando disponível, com queda para camada em memória em implantação de instância única.</t>
+          <t>Restrito às oportunidades da própria organização. A organização não participa do fórum: publica ações, acompanha inscrições e emite certificados.</t>
         </is>
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -3533,12 +3533,12 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-002</t>
+          <t>RF-NOT-001</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Listar notificações</t>
+          <t>Entregar notificação em tempo real</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
@@ -3548,17 +3548,17 @@
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>Usuário vê o histórico de avisos e quantos estão por ler.</t>
+          <t>O aviso chega sem recarregar a página.</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>GET /api/notificacoes/ e /nao-lidas/.</t>
+          <t>WebSocket em /ws/notificacoes/ com Django Channels sobre Daphne. Sala por usuário. Camada em Redis quando disponível, com queda para camada em memória em implantação de instância única.</t>
         </is>
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -3573,12 +3573,12 @@
       </c>
       <c r="B75" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-003</t>
+          <t>RF-NOT-002</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Marcar notificação como lida</t>
+          <t>Listar notificações</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
@@ -3588,12 +3588,12 @@
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Usuário marca um aviso ou todos de uma vez.</t>
+          <t>Usuário vê o histórico de avisos e quantos estão por ler.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>POST /api/notificacoes/{id}/marcar-lida/ e /marcar-todas-lidas/.</t>
+          <t>GET /api/notificacoes/ e /nao-lidas/.</t>
         </is>
       </c>
       <c r="G75" s="9" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="H75" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3613,12 +3613,12 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-004</t>
+          <t>RF-NOT-003</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Limpar notificações</t>
+          <t>Marcar notificação como lida</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
@@ -3628,12 +3628,12 @@
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>Usuário descarta os avisos já lidos.</t>
+          <t>Usuário marca um aviso ou todos de uma vez.</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>POST /api/notificacoes/limpar/.</t>
+          <t>POST /api/notificacoes/{id}/marcar-lida/ e /marcar-todas-lidas/.</t>
         </is>
       </c>
       <c r="G76" s="8" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>DESEJÁVEL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -3653,12 +3653,12 @@
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-005</t>
+          <t>RF-NOT-004</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Agrupar aviso por conversa</t>
+          <t>Limpar notificações</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -3668,22 +3668,22 @@
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Uma conversa com muitas mensagens novas gera um aviso, e não um por mensagem.</t>
+          <t>Usuário descarta os avisos já lidos.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Enquanto houver aviso não lido daquela conversa, não se cria outro. Sem isso, uma discussão ativa produziria dezenas de avisos e a pessoa desligaria todos.</t>
+          <t>POST /api/notificacoes/limpar/.</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H77" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -3693,37 +3693,37 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>RF-PRF-001</t>
+          <t>RF-NOT-005</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Visualizar perfil</t>
+          <t>Agrupar aviso por conversa</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>Perfil</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>Usuário vê seus dados, foto, curso, período e disciplinas.</t>
+          <t>Uma conversa com muitas mensagens novas gera um aviso, e não um por mensagem.</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>Compõe dados de /api/auth/me/ com o andamento por disciplina.</t>
+          <t>Enquanto houver aviso não lido daquela conversa, não se cria outro. Sem isso, uma discussão ativa produziria dezenas de avisos e a pessoa desligaria todos.</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -3733,12 +3733,12 @@
       </c>
       <c r="B79" s="9" t="inlineStr">
         <is>
-          <t>RF-PRF-002</t>
+          <t>RF-PRF-001</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Consultar histórico de participação</t>
+          <t>Visualizar perfil</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
@@ -3748,12 +3748,12 @@
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê suas publicações, inscrições e certificados reunidos.</t>
+          <t>Usuário vê seus dados, foto, curso, período e disciplinas.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Agrega as consultas de cada módulo na tela de perfil.</t>
+          <t>Compõe dados de /api/auth/me/ com o andamento por disciplina.</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="H79" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3773,37 +3773,37 @@
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>RF-COO-001</t>
+          <t>RF-PRF-002</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Acompanhar o curso por disciplina</t>
+          <t>Consultar histórico de participação</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Perfil</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>A coordenação vê o movimento de cada disciplina do curso: volume de dúvidas, proporção respondida e tempo até a primeira resposta.</t>
+          <t>Usuário vê suas publicações, inscrições e certificados reunidos.</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>Painel que agrega por disciplina e período. Identifica disciplina com muita dúvida sem resposta, que é o sinal que o painel existe para produzir.</t>
+          <t>Agrega as consultas de cada módulo na tela de perfil.</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -3813,12 +3813,12 @@
       </c>
       <c r="B81" s="9" t="inlineStr">
         <is>
-          <t>RF-COO-002</t>
+          <t>RF-COO-001</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>Detalhar uma disciplina</t>
+          <t>Acompanhar o curso por disciplina</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
@@ -3828,12 +3828,12 @@
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>A coordenação abre uma disciplina e vê as dúvidas mais vistas e as sem resposta.</t>
+          <t>A coordenação vê o movimento de cada disciplina do curso: volume de dúvidas, proporção respondida e tempo até a primeira resposta.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Consulta por disciplina, ordenada pela razão entre visualizações e respostas.</t>
+          <t>Painel que agrega por disciplina e período. Identifica disciplina com muita dúvida sem resposta, que é o sinal que o painel existe para produzir.</t>
         </is>
       </c>
       <c r="G81" s="9" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="H81" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3853,12 +3853,12 @@
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>RF-COO-003</t>
+          <t>RF-COO-002</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Importar a matriz curricular</t>
+          <t>Detalhar uma disciplina</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr">
@@ -3868,12 +3868,12 @@
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>As disciplinas do curso entram na plataforma a partir do projeto pedagógico.</t>
+          <t>A coordenação abre uma disciplina e vê as dúvidas mais vistas e as sem resposta.</t>
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>Comando importar_matriz_ppc, que lê o ementário e cadastra código, nome, período e carga horária. A paridade do período define o semestre de oferta.</t>
+          <t>Consulta por disciplina, ordenada pela razão entre visualizações e respostas.</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
@@ -3893,32 +3893,32 @@
       </c>
       <c r="B83" s="9" t="inlineStr">
         <is>
-          <t>RF-AUD-001</t>
+          <t>RF-COO-003</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>Registrar ações sensíveis</t>
+          <t>Importar a matriz curricular</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Coordenação</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Ações de moderação e de gestão de vínculos ficam registradas.</t>
+          <t>As disciplinas do curso entram na plataforma a partir do projeto pedagógico.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Modelo de registro de auditoria, com autor, ação, alvo e momento. Consulta restrita à administração.</t>
+          <t>Comando importar_matriz_ppc, que lê o ementário e cadastra código, nome, período e carga horária. A paridade do período define o semestre de oferta.</t>
         </is>
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Coordenação</t>
         </is>
       </c>
       <c r="H83" s="9" t="inlineStr">
@@ -3933,32 +3933,32 @@
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>RF-SIS-001</t>
+          <t>RF-AUD-001</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Alternar entre tema claro e escuro</t>
+          <t>Registrar ações sensíveis</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
         <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>Ações de moderação e de gestão de vínculos ficam registradas.</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>Modelo de registro de auditoria, com autor, ação, alvo e momento. Consulta restrita à administração.</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
           <t>Sistema</t>
-        </is>
-      </c>
-      <c r="E84" s="8" t="inlineStr">
-        <is>
-          <t>Usuário escolhe o tema e a escolha permanece entre visitas.</t>
-        </is>
-      </c>
-      <c r="F84" s="8" t="inlineStr">
-        <is>
-          <t>Alternância por variáveis de cor no navegador, com a preferência guardada localmente. Todas as cores da interface vêm dessas variáveis: valor fixo escrito no código produz texto ilegível num dos dois temas.</t>
-        </is>
-      </c>
-      <c r="G84" s="8" t="inlineStr">
-        <is>
-          <t>Todos</t>
         </is>
       </c>
       <c r="H84" s="8" t="inlineStr">
@@ -3973,12 +3973,12 @@
       </c>
       <c r="B85" s="9" t="inlineStr">
         <is>
-          <t>RF-SIS-002</t>
+          <t>RF-SIS-001</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>Consultar a documentação da API</t>
+          <t>Alternar entre tema claro e escuro</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
@@ -3988,17 +3988,17 @@
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>A especificação da API fica acessível e navegável.</t>
+          <t>Usuário escolhe o tema e a escolha permanece entre visitas.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Esquema OpenAPI gerado por drf-spectacular a partir das views e serializadores, com interface de navegação.</t>
+          <t>Alternância por variáveis de cor no navegador, com a preferência guardada localmente. Todas as cores da interface vêm dessas variáveis: valor fixo escrito no código produz texto ilegível num dos dois temas.</t>
         </is>
       </c>
       <c r="G85" s="9" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H85" s="9" t="inlineStr">
@@ -4013,42 +4013,82 @@
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
+          <t>RF-SIS-002</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Consultar a documentação da API</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>A especificação da API fica acessível e navegável.</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>Esquema OpenAPI gerado por drf-spectacular a partir das views e serializadores, com interface de navegação.</t>
+        </is>
+      </c>
+      <c r="G86" s="8" t="inlineStr">
+        <is>
+          <t>Desenvolvedor</t>
+        </is>
+      </c>
+      <c r="H86" s="8" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="9" t="inlineStr">
+        <is>
           <t>RF-SIS-003</t>
         </is>
       </c>
-      <c r="C86" s="8" t="inlineStr">
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>Carregar dados de demonstração</t>
         </is>
       </c>
-      <c r="D86" s="8" t="inlineStr">
+      <c r="D87" s="9" t="inlineStr">
         <is>
           <t>Sistema</t>
         </is>
       </c>
-      <c r="E86" s="8" t="inlineStr">
+      <c r="E87" s="9" t="inlineStr">
         <is>
           <t>A plataforma pode ser povoada com um semestre completo para demonstração e avaliação.</t>
         </is>
       </c>
-      <c r="F86" s="8" t="inlineStr">
+      <c r="F87" s="9" t="inlineStr">
         <is>
           <t>Comando popular_demonstracao, com semente fixa para que a mesma execução produza sempre o mesmo conjunto. Gera disciplinas com ritmos distintos de atividade, deliberadamente incluindo uma sem professor atribuído, para que o painel de coordenação tenha o que apontar.</t>
         </is>
       </c>
-      <c r="G86" s="8" t="inlineStr">
+      <c r="G87" s="9" t="inlineStr">
         <is>
           <t>Coordenação</t>
         </is>
       </c>
-      <c r="H86" s="8" t="inlineStr">
+      <c r="H87" s="9" t="inlineStr">
         <is>
           <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H86"/>
+  <autoFilter ref="A1:H87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revisa os requisitos contra o código e reorganiza o README
RF passam de 86 para 97 e RNF de 51 para 59, com divergências do TCC1 ampliadas e aba de lacunas conhecidas. O README corrige o endereço de implantação, a URL de clone e a rota da API, e o schema.yml é regenerado. Só documentação.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
+++ b/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Divergências TCC1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos Funcionais'!$A$1:$H$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Divergências TCC1'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Requisitos Funcionais'!$A$1:$H$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Divergências TCC1'!$A$1:$E$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -507,7 +507,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Levantamento a partir do sistema implementado, e não do planejamento. As diferenças em relação ao TCC1 estão registradas na aba Divergências TCC1, com a justificativa de cada uma.</t>
+          <t>Levantamento a partir do sistema implementado, e não do planejamento. As diferenças em relação ao TCC1 estão registradas na aba Divergências TCC1, com a justificativa de cada uma. Revisado em 24/10/2026 contra o código (v1.1.2).</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H87,"CRÍTICA")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H98,"CRÍTICA")</f>
         <v/>
       </c>
     </row>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H87,"ESSENCIAL")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H98,"ESSENCIAL")</f>
         <v/>
       </c>
     </row>
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H87,"IMPORTANTE")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H98,"IMPORTANTE")</f>
         <v/>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF('Requisitos Funcionais'!H2:H87,"DESEJÁVEL")</f>
+        <f>COUNTIF('Requisitos Funcionais'!H2:H98,"DESEJÁVEL")</f>
         <v/>
       </c>
     </row>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTA('Requisitos Funcionais'!B2:B87)</f>
+        <f>COUNTA('Requisitos Funcionais'!B2:B98)</f>
         <v/>
       </c>
     </row>
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2013,37 +2013,37 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-001</t>
+          <t>RF-FOR-024</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Propor trabalho em grupo</t>
+          <t>Limitar a uma monitoria por disciplina</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>Colaboração</t>
+          <t>Fórum</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Professor cria um trabalho definindo quantidade de grupos, tamanho máximo, prazo e forma de montagem.</t>
+          <t>A disciplina tem um monitor por vez, e atribuir outro exige encerrar a monitoria atual.</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/. Exige que a pessoa lecione a disciplina — a coordenação não passa nesta verificação, porque supervisionar não é participar da turma.</t>
+          <t>Verificação na criação do vínculo de disciplina (PermissaoDisciplinaViewSet.create). Se já houver monitor ativo, responde 400 com mensagem que cita o monitor atual e orienta a encerrar a monitoria antes. A regra existe porque a monitoria é um encargo único por turma, e sem ela o canal da monitoria e a fila de pedidos de ajuda alcançariam quem já não atende.</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Professor/Coordenação</t>
         </is>
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2053,37 +2053,37 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-002</t>
+          <t>RF-FOR-025</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Anexar material ao enunciado</t>
+          <t>Sanear vínculos com disciplinas</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Colaboração</t>
+          <t>Fórum</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>Professor anexa a especificação, a base de dados e o esqueleto de código ao próprio trabalho.</t>
+          <t>A coordenação identifica e corrige inconsistências nos vínculos, como disciplina com vários monitores ou pessoas homônimas com papéis repetidos.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/{id}/anexar/ e remoção correspondente. Lista de tipos aceitos e limite de tamanho no servidor. Fica no trabalho, e não no grupo: é material da turma inteira. Sem este espaço, o professor distribuiria por outro canal e o enunciado ficaria separado dos arquivos.</t>
+          <t>Comando sanear_vinculos. Sem argumento apenas relata. Com --aplicar corrige o que é seguro e reversível (desativa o monitor excedente) e apenas relata o que exige decisão humana, como decidir qual de dois cadastros homônimos é a pessoa real.</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Coordenação</t>
         </is>
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -2093,37 +2093,37 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-003</t>
+          <t>RF-FOR-026</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Criar grupos vazios</t>
+          <t>Indexar publicações para a busca semântica</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Colaboração</t>
+          <t>Fórum</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Sistema gera os grupos previstos para que os alunos escolham onde entrar.</t>
+          <t>A busca por significado passa a incluir o conteúdo que já existia antes de o recurso ser ligado.</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/{id}/criar-grupos/. Cria a conversa privada de cada grupo junto.</t>
+          <t>Comando indexar_forum (--tudo refaz todos os vetores, --lote define o tamanho). Necessário ao ligar a busca num banco com conteúdo, ao trocar o modelo de representação e após importações que não passaram pelos sinais. Processa em lote por ser muito mais barato que um a um.</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Coordenação</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2133,12 +2133,12 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-004</t>
+          <t>RF-COL-001</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Sortear a composição dos grupos</t>
+          <t>Propor trabalho em grupo</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -2148,12 +2148,12 @@
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Distribuição aleatória dos matriculados entre os grupos.</t>
+          <t>Professor cria um trabalho definindo quantidade de grupos, tamanho máximo, prazo e forma de montagem.</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/{id}/sortear/. Respeita o tamanho máximo e sincroniza os participantes das conversas.</t>
+          <t>POST /api/colaboracao/trabalhos/. Exige que a pessoa lecione a disciplina — a coordenação não passa nesta verificação, porque supervisionar não é participar da turma.</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="H39" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -2173,12 +2173,12 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-005</t>
+          <t>RF-COL-002</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Entrar em grupo</t>
+          <t>Anexar material ao enunciado</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -2188,17 +2188,17 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Aluno escolhe o grupo de que quer participar.</t>
+          <t>Professor anexa a especificação, a base de dados e o esqueleto de código ao próprio trabalho.</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/grupos/{id}/entrar/. Recusa se o grupo estiver cheio ou se a pessoa já estiver em outro grupo do mesmo trabalho. Insere na conversa do grupo.</t>
+          <t>POST /api/colaboracao/trabalhos/{id}/anexar/ e remoção correspondente. Lista de tipos aceitos e limite de tamanho no servidor. Fica no trabalho, e não no grupo: é material da turma inteira. Sem este espaço, o professor distribuiria por outro canal e o enunciado ficaria separado dos arquivos.</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr">
@@ -2213,12 +2213,12 @@
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-006</t>
+          <t>RF-COL-003</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Sair de grupo</t>
+          <t>Criar grupos vazios</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -2228,22 +2228,22 @@
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Aluno deixa o grupo, com confirmação antes.</t>
+          <t>Sistema gera os grupos previstos para que os alunos escolham onde entrar.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/grupos/{id}/sair/. Remove da conversa e atualiza a contagem de participantes.</t>
+          <t>POST /api/colaboracao/trabalhos/{id}/criar-grupos/. Cria a conversa privada de cada grupo junto.</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2253,12 +2253,12 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-007</t>
+          <t>RF-COL-004</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Definir responsável pelo grupo</t>
+          <t>Sortear a composição dos grupos</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -2268,22 +2268,22 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>O grupo indica quem responde por ele.</t>
+          <t>Distribuição aleatória dos matriculados entre os grupos.</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/grupos/{id}/definir-lider/.</t>
+          <t>POST /api/colaboracao/trabalhos/{id}/sortear/. Respeita o tamanho máximo e sincroniza os participantes das conversas.</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>Aluno/Professor</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>DESEJÁVEL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2293,12 +2293,12 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-008</t>
+          <t>RF-COL-005</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Conversar em tempo real no grupo</t>
+          <t>Entrar em grupo</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
@@ -2308,12 +2308,12 @@
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>Os integrantes trocam mensagens, imagens, documentos e áudio no espaço privado do grupo.</t>
+          <t>Aluno escolhe o grupo de que quer participar.</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>GET e POST /api/colaboracao/conversas/{id}/mensagens/, com entrega imediata por WebSocket via Django Channels. A conversa é privada aos integrantes, inclusive em relação ao professor. É a decisão que sustenta o módulo: sem privacidade, os grupos migram para aplicativos externos e o material se perde no fim do semestre.</t>
+          <t>POST /api/colaboracao/grupos/{id}/entrar/. Recusa se o grupo estiver cheio ou se a pessoa já estiver em outro grupo do mesmo trabalho. Insere na conversa do grupo.</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2333,12 +2333,12 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-009</t>
+          <t>RF-COL-006</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Excluir mensagem enviada</t>
+          <t>Sair de grupo</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -2348,17 +2348,17 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>Autor apaga uma mensagem dentro de um prazo curto após o envio.</t>
+          <t>Aluno deixa o grupo, com confirmação antes.</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>DELETE /api/colaboracao/mensagens/{id}/. Janela de três minutos, verificação de autoria e exclusão lógica. Recusa se a mensagem já tiver originado um pedido de ajuda, para não apagar o que já foi encaminhado a terceiros. Anuncia a exclusão aos demais pelo WebSocket.</t>
+          <t>POST /api/colaboracao/grupos/{id}/sair/. Remove da conversa e atualiza a contagem de participantes.</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>Autor</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H44" s="8" t="inlineStr">
@@ -2373,12 +2373,12 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-010</t>
+          <t>RF-COL-007</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Registrar leitura da conversa</t>
+          <t>Definir responsável pelo grupo</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
@@ -2388,22 +2388,22 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>O contador de mensagens não lidas zera quando a pessoa abre a conversa.</t>
+          <t>O grupo indica quem responde por ele.</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/conversas/{id}/marcar-lida/. O marcador fica no participante, e não na mensagem: guardar um registro por mensagem e por pessoa inviabilizaria qualquer conversa ativa.</t>
+          <t>POST /api/colaboracao/grupos/{id}/definir-lider/.</t>
         </is>
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Aluno/Professor</t>
         </is>
       </c>
       <c r="H45" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -2413,12 +2413,12 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-011</t>
+          <t>RF-COL-008</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Encaminhar dúvida do grupo</t>
+          <t>Conversar em tempo real no grupo</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>O grupo marca uma mensagem e a encaminha a quem conduz a turma, com uma descrição do problema.</t>
+          <t>Os integrantes trocam mensagens, imagens, documentos e áudio no espaço privado do grupo.</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/conversas/{id}/pedir-ajuda/. O destino é decidido pelo sistema: monitoria quando a disciplina tem monitor, professor quando não tem. Só a mensagem marcada e a descrição atravessam — a conversa em volta continua invisível.</t>
+          <t>GET e POST /api/colaboracao/conversas/{id}/mensagens/, com entrega imediata por WebSocket via Django Channels. A conversa é privada aos integrantes, inclusive em relação ao professor. É a decisão que sustenta o módulo: sem privacidade, os grupos migram para aplicativos externos e o material se perde no fim do semestre.</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -2453,12 +2453,12 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-012</t>
+          <t>RF-COL-009</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Assumir pedido de ajuda</t>
+          <t>Excluir mensagem enviada</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
@@ -2468,17 +2468,17 @@
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>Monitor ou professor assume o atendimento.</t>
+          <t>Autor apaga uma mensagem dentro de um prazo curto após o envio.</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/ajuda/{id}/assumir/. Evita que dois atendam o mesmo pedido.</t>
+          <t>DELETE /api/colaboracao/mensagens/{id}/. Janela de três minutos, verificação de autoria e exclusão lógica. Recusa se a mensagem já tiver originado um pedido de ajuda, para não apagar o que já foi encaminhado a terceiros. Anuncia a exclusão aos demais pelo WebSocket.</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>Monitor/Professor</t>
+          <t>Autor</t>
         </is>
       </c>
       <c r="H47" s="9" t="inlineStr">
@@ -2493,12 +2493,12 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-013</t>
+          <t>RF-COL-010</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Responder pedido de ajuda</t>
+          <t>Registrar leitura da conversa</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
@@ -2508,22 +2508,22 @@
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>Quem assumiu responde e a resposta chega ao grupo.</t>
+          <t>O contador de mensagens não lidas zera quando a pessoa abre a conversa.</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/ajuda/{id}/responder/. Registra a resposta e notifica os integrantes.</t>
+          <t>POST /api/colaboracao/conversas/{id}/marcar-lida/. O marcador fica no participante, e não na mensagem: guardar um registro por mensagem e por pessoa inviabilizaria qualquer conversa ativa.</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>Monitor/Professor</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2533,12 +2533,12 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-014</t>
+          <t>RF-COL-011</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Reunir arquivos por disciplina</t>
+          <t>Encaminhar dúvida do grupo</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
@@ -2548,22 +2548,22 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Usuário encontra num lugar só todo o material que passou por ele, separado por matéria.</t>
+          <t>O grupo marca uma mensagem e a encaminha a quem conduz a turma, com uma descrição do problema.</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/arquivos/. Reúne três origens: anexo de conversa, material de trabalho e anexo de publicação. Sem modelo novo e sem cópia: a consulta lê o que já está gravado, mantendo o recorte de permissão de cada origem. Anexo de conversa só aparece para quem participa dela.</t>
+          <t>POST /api/colaboracao/conversas/{id}/pedir-ajuda/. O destino é decidido pelo sistema: monitoria quando a disciplina tem monitor, professor quando não tem. Só a mensagem marcada e a descrição atravessam — a conversa em volta continua invisível.</t>
         </is>
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>Aluno/Monitor/Professor</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -2573,12 +2573,12 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-015</t>
+          <t>RF-COL-012</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Consultar trabalhos da disciplina</t>
+          <t>Assumir pedido de ajuda</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -2588,22 +2588,22 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>Usuário vê os trabalhos propostos, o prazo e a situação do próprio grupo.</t>
+          <t>Monitor ou professor assume o atendimento.</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/trabalhos/. Filtra pelas disciplinas de vínculo. Quem não tem vínculo com nenhuma disciplina não alcança esta tela: a aba sequer aparece, porque toda ação disponível ali terminaria em erro.</t>
+          <t>POST /api/colaboracao/ajuda/{id}/assumir/. Evita que dois atendam o mesmo pedido.</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Aluno/Monitor/Professor</t>
+          <t>Monitor/Professor</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2613,12 +2613,12 @@
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-016</t>
+          <t>RF-COL-013</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Consultar composição dos grupos</t>
+          <t>Responder pedido de ajuda</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
@@ -2628,17 +2628,17 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Quem conduz a turma vê como os grupos ficaram formados.</t>
+          <t>Quem assumiu responde e a resposta chega ao grupo.</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/grupos/. O professor enxerga a composição e o andamento, mas não entra na conversa privada da equipe.</t>
+          <t>POST /api/colaboracao/ajuda/{id}/responder/. Registra a resposta e notifica os integrantes.</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Monitor/Professor</t>
         </is>
       </c>
       <c r="H51" s="9" t="inlineStr">
@@ -2653,12 +2653,12 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>RF-COL-017</t>
+          <t>RF-COL-014</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Listar conversas com pendências</t>
+          <t>Reunir arquivos por disciplina</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -2668,12 +2668,12 @@
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>Usuário vê suas conversas com a quantidade de mensagens por ler.</t>
+          <t>Usuário encontra num lugar só todo o material que passou por ele, separado por matéria.</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/conversas/. Filtra por participação e calcula as não lidas a partir do marcador de leitura de cada participante.</t>
+          <t>GET /api/colaboracao/arquivos/. Reúne três origens: anexo de conversa, material de trabalho e anexo de publicação. Sem modelo novo e sem cópia: a consulta lê o que já está gravado, mantendo o recorte de permissão de cada origem. Anexo de conversa só aparece para quem participa dela.</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2693,12 +2693,12 @@
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>RF-COL-018</t>
+          <t>RF-COL-015</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Acompanhar a fila de pedidos de ajuda</t>
+          <t>Consultar trabalhos da disciplina</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
@@ -2708,17 +2708,17 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Quem conduz a turma vê os pedidos abertos, em atendimento e resolvidos.</t>
+          <t>Usuário vê os trabalhos propostos, o prazo e a situação do próprio grupo.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>GET /api/colaboracao/ajuda/. O destino do pedido decide quem o enxerga: monitoria quando a disciplina tem monitor, professor quando não tem.</t>
+          <t>GET /api/colaboracao/trabalhos/. Filtra pelas disciplinas de vínculo. Quem não tem vínculo com nenhuma disciplina não alcança esta tela: a aba sequer aparece, porque toda ação disponível ali terminaria em erro.</t>
         </is>
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>Monitor/Professor</t>
+          <t>Aluno/Monitor/Professor</t>
         </is>
       </c>
       <c r="H53" s="9" t="inlineStr">
@@ -2733,32 +2733,32 @@
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-001</t>
+          <t>RF-COL-016</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Publicar oportunidade</t>
+          <t>Consultar composição dos grupos</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>Voluntariado</t>
+          <t>Colaboração</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>Organização parceira cadastra uma ação de voluntariado com período, vagas, carga horária e local.</t>
+          <t>Quem conduz a turma vê como os grupos ficaram formados.</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/oportunidades/. Restrito ao perfil de organização.</t>
+          <t>GET /api/colaboracao/grupos/. O professor enxerga a composição e o andamento, mas não entra na conversa privada da equipe.</t>
         </is>
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
@@ -2773,32 +2773,32 @@
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-002</t>
+          <t>RF-COL-017</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Consultar oportunidades</t>
+          <t>Listar conversas com pendências</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Voluntariado</t>
+          <t>Colaboração</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Estudante vê as ações disponíveis, com filtro por situação e busca por texto.</t>
+          <t>Usuário vê suas conversas com a quantidade de mensagens por ler.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>GET /api/voluntariado/oportunidades/. Informa vagas preenchidas e total.</t>
+          <t>GET /api/colaboracao/conversas/. Filtra por participação e calcula as não lidas a partir do marcador de leitura de cada participante.</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Aluno/Monitor/Professor</t>
         </is>
       </c>
       <c r="H55" s="9" t="inlineStr">
@@ -2813,32 +2813,32 @@
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-003</t>
+          <t>RF-COL-018</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Inscrever-se em oportunidade</t>
+          <t>Acompanhar a fila de pedidos de ajuda</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>Voluntariado</t>
+          <t>Colaboração</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>Estudante se candidata a uma vaga.</t>
+          <t>Quem conduz a turma vê os pedidos abertos, em atendimento e resolvidos.</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/oportunidades/{id}/inscrever/. Unicidade por par pessoa e oportunidade. Verifica vaga disponível dentro de transação, para que duas inscrições simultâneas não ultrapassem o limite.</t>
+          <t>GET /api/colaboracao/ajuda/. O destino do pedido decide quem o enxerga: monitoria quando a disciplina tem monitor, professor quando não tem.</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Monitor/Professor</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
@@ -2853,32 +2853,32 @@
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-004</t>
+          <t>RF-COL-019</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Desistir da inscrição</t>
+          <t>Canal da monitoria por disciplina</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Voluntariado</t>
+          <t>Colaboração</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Estudante cancela a própria inscrição e libera a vaga.</t>
+          <t>Professor e monitor de cada disciplina ganham uma conversa reservada a eles, para alinhar o atendimento aos alunos.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/inscricoes/{id}/desistir/.</t>
+          <t>Conversa do tipo "monitoria", criada por sinal ao atribuir o monitor (transaction.on_commit). Participantes: os professores e o monitor ativo daquela disciplina. Aluno não entra, professor ou monitor de outra disciplina não a enxerga, e disciplina sem monitor não ganha canal. Título "Monitoria de &lt;código&gt;".</t>
         </is>
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H57" s="9" t="inlineStr">
@@ -2893,37 +2893,37 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-005</t>
+          <t>RF-COL-020</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Aprovar ou rejeitar inscrição</t>
+          <t>Arquivar o canal ao fim da monitoria</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>Voluntariado</t>
+          <t>Colaboração</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>A organização decide quem participa.</t>
+          <t>Quando a monitoria termina, o histórico permanece, mas o canal deixa de aceitar mensagens.</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/inscricoes/{id}/aprovar/ e rejeitar. Notifica o candidato da decisão.</t>
+          <t>O fim do vínculo marca a conversa como somente leitura (arquivada_em). Se a monitoria for reconstituída, o mesmo canal reabre. O histórico é preservado para consulta.</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -2933,37 +2933,37 @@
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-006</t>
+          <t>RF-COL-021</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Remover participante</t>
+          <t>Indicar presença na conversa</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Voluntariado</t>
+          <t>Colaboração</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>A organização retira alguém já aprovado.</t>
+          <t>Os participantes veem quantas pessoas estão conectadas à conversa naquele momento.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/inscricoes/{id}/remover/. Devolve a vaga.</t>
+          <t>WebSocket /ws/conversas/{id}/ (ConversaConsumer). Contagem mantida em memória por conversa e anunciada ao grupo a cada entrada ou saída, no formato {tipo: presenca, conectados: n}. É informação efêmera e se perde ao reiniciar o processo, por isso não é gravada no banco.</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno/Monitor/Professor</t>
         </is>
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -2973,37 +2973,37 @@
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-007</t>
+          <t>RF-COL-022</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Concluir participação</t>
+          <t>Consultar participantes da conversa</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>Voluntariado</t>
+          <t>Colaboração</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t>A organização confirma que a pessoa cumpriu a ação, o que dispara a emissão do certificado.</t>
+          <t>Usuário vê quem faz parte de uma conversa de que participa.</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>POST /api/voluntariado/inscricoes/{id}/concluir/. Registra a conclusão e gera o certificado na sequência.</t>
+          <t>GET /api/colaboracao/conversas/{id}/participantes/. Restrito a quem participa da conversa.</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno/Monitor/Professor</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -3013,12 +3013,12 @@
       </c>
       <c r="B61" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-008</t>
+          <t>RF-VOL-001</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Emitir certificado em PDF</t>
+          <t>Publicar oportunidade</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
@@ -3028,22 +3028,22 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Certificado de participação com código de verificação, para aproveitamento das horas como atividade complementar.</t>
+          <t>Organização parceira cadastra uma ação de voluntariado com período, vagas, carga horária e local.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>Geração com WeasyPrint a partir de modelo HTML, com identidade visual da UNIFEI, dados da ação, carga horária e código único de conferência.</t>
+          <t>POST /api/voluntariado/oportunidades/. Restrito ao perfil de organização.</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3053,12 +3053,12 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-009</t>
+          <t>RF-VOL-002</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>Consultar certificados</t>
+          <t>Consultar oportunidades</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
@@ -3068,12 +3068,12 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>Estudante acessa e baixa os certificados que recebeu.</t>
+          <t>Estudante vê as ações disponíveis, com filtro por situação e busca por texto.</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>GET /api/voluntariado/certificados/.</t>
+          <t>GET /api/voluntariado/oportunidades/. Informa vagas preenchidas e total.</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
@@ -3093,12 +3093,12 @@
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-010</t>
+          <t>RF-VOL-003</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Acompanhar inscritos</t>
+          <t>Inscrever-se em oportunidade</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -3108,17 +3108,17 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>A organização vê quem se inscreveu e em que situação está cada inscrição.</t>
+          <t>Estudante se candidata a uma vaga.</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>GET /api/voluntariado/oportunidades/{id}/inscricoes/.</t>
+          <t>POST /api/voluntariado/oportunidades/{id}/inscrever/. Unicidade por par pessoa e oportunidade. Verifica vaga disponível dentro de transação, para que duas inscrições simultâneas não ultrapassem o limite.</t>
         </is>
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H63" s="9" t="inlineStr">
@@ -3133,12 +3133,12 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-011</t>
+          <t>RF-VOL-004</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>Editar oportunidade publicada</t>
+          <t>Desistir da inscrição</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
@@ -3148,17 +3148,17 @@
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>A organização corrige dados da ação já publicada.</t>
+          <t>Estudante cancela a própria inscrição e libera a vaga.</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>PUT /api/voluntariado/oportunidades/{id}/. Verifica que a organização é a autora. Alteração de data notifica os inscritos.</t>
+          <t>POST /api/voluntariado/inscricoes/{id}/desistir/.</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
@@ -3173,12 +3173,12 @@
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-012</t>
+          <t>RF-VOL-005</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Encerrar oportunidade</t>
+          <t>Aprovar ou rejeitar inscrição</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>A organização encerra as inscrições sem apagar o registro.</t>
+          <t>A organização decide quem participa.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Alteração de situação, e não remoção. Quem participou precisa de um caminho de volta até a ação para alcançar o certificado.</t>
+          <t>POST /api/voluntariado/inscricoes/{id}/aprovar/ e rejeitar. Notifica o candidato da decisão.</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr">
@@ -3213,12 +3213,12 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-013</t>
+          <t>RF-VOL-006</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>Consultar as próprias inscrições</t>
+          <t>Remover participante</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
@@ -3228,22 +3228,22 @@
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>Estudante acompanha em que situação está cada candidatura.</t>
+          <t>A organização retira alguém já aprovado.</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>GET /api/voluntariado/inscricoes/minhas/.</t>
+          <t>POST /api/voluntariado/inscricoes/{id}/remover/. Devolve a vaga.</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -3253,12 +3253,12 @@
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-014</t>
+          <t>RF-VOL-007</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>Publicar campanha de doação</t>
+          <t>Concluir participação</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -3268,12 +3268,12 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>A organização cadastra uma arrecadação de itens, como agasalhos ou alimentos, definindo como a contribuição será contada.</t>
+          <t>A organização confirma que a pessoa cumpriu a ação, o que dispara a emissão do certificado.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>Modalidade da oportunidade. A unidade é texto livre — peças de agasalho, quilos de alimento — porque qualquer lista fixa não teria a categoria da próxima campanha. Meta é opcional. Vagas e carga horária não se aplicam: campanha não limita participantes nem cumpre hora.</t>
+          <t>POST /api/voluntariado/inscricoes/{id}/concluir/. Registra a conclusão e gera o certificado na sequência.</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="H67" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -3293,12 +3293,12 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-015</t>
+          <t>RF-VOL-008</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Declarar doação</t>
+          <t>Emitir certificado em PDF</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
@@ -3308,22 +3308,22 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>Estudante informa quanto pretende entregar à campanha.</t>
+          <t>Certificado de participação com código de verificação, para aproveitamento das horas como atividade complementar.</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>POST em inscrever, com quantidade declarada e descrição opcional do item. É declaração de intenção: o valor fica registrado à parte e não entra na contagem da campanha até a organização confirmar o recebimento.</t>
+          <t>Geração com WeasyPrint a partir de modelo HTML, com identidade visual da UNIFEI, dados da ação, carga horária e código único de conferência.</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Aluno</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -3333,12 +3333,12 @@
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-016</t>
+          <t>RF-VOL-009</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Confirmar recebimento da doação</t>
+          <t>Consultar certificados</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -3348,22 +3348,22 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>A organização registra quanto de fato recebeu, que pode divergir do que foi declarado.</t>
+          <t>Estudante acessa e baixa os certificados que recebeu.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>POST em concluir, com a quantidade confirmada. Sem valor informado, vale o declarado. O campo é somente leitura para o estudante: se ele pudesse registrar o próprio recebimento, o total da campanha deixaria de significar algo. Emite o certificado na mesma operação.</t>
+          <t>GET /api/voluntariado/certificados/.</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H69" s="9" t="inlineStr">
         <is>
-          <t>CRÍTICA</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3373,12 +3373,12 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>RF-VOL-017</t>
+          <t>RF-VOL-010</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Acompanhar a arrecadação</t>
+          <t>Acompanhar inscritos</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
@@ -3388,17 +3388,17 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>A página da campanha mostra quanto já foi arrecadado e, havendo meta, o progresso em relação a ela.</t>
+          <t>A organização vê quem se inscreveu e em que situação está cada inscrição.</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>Soma apenas as quantidades confirmadas em participações concluídas. Sem meta declarada não há barra de progresso: a barra precisa de um denominador, e inventar um faria a campanha parecer mais adiantada do que está.</t>
+          <t>GET /api/voluntariado/oportunidades/{id}/inscricoes/.</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H70" s="8" t="inlineStr">
@@ -3413,12 +3413,12 @@
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>RF-VOL-018</t>
+          <t>RF-VOL-011</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Certificar participação em campanha</t>
+          <t>Editar oportunidade publicada</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -3428,22 +3428,22 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Quem doou recebe certificado declarando a contribuição.</t>
+          <t>A organização corrige dados da ação já publicada.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>O texto do certificado muda com a modalidade: registra o que foi entregue e acrescenta que a organização atribui àquela participação o equivalente a um número de horas por ela definido. A formulação é deliberada — doar não é cumprir hora, e quem receber o documento precisa saber que avalia uma equivalência declarada pela entidade.</t>
+          <t>PUT /api/voluntariado/oportunidades/{id}/. Verifica que a organização é a autora. Alteração de data notifica os inscritos.</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>ESSENCIAL</t>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
@@ -3453,32 +3453,32 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>RF-PAI-001</t>
+          <t>RF-VOL-012</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Painel de quem conduz a turma</t>
+          <t>Encerrar oportunidade</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>Painéis</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>Professor e monitor veem, num lugar só, as dúvidas sem resposta, os pedidos de ajuda abertos e os trabalhos em andamento das suas turmas.</t>
+          <t>A organização encerra as inscrições sem apagar o registro.</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>Composição das consultas dos módulos, restrita às disciplinas em que a pessoa leciona ou exerce monitoria. O monitor vê apenas onde é monitor.</t>
+          <t>Alteração de situação, e não remoção. Quem participou precisa de um caminho de volta até a ação para alcançar o certificado.</t>
         </is>
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -3493,32 +3493,32 @@
       </c>
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>RF-PAI-002</t>
+          <t>RF-VOL-013</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Painel da organização parceira</t>
+          <t>Consultar as próprias inscrições</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Painéis</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>A organização vê suas oportunidades, quantos se inscreveram e quantos concluíram.</t>
+          <t>Estudante acompanha em que situação está cada candidatura.</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>Restrito às oportunidades da própria organização. A organização não participa do fórum: publica ações, acompanha inscrições e emite certificados.</t>
+          <t>GET /api/voluntariado/inscricoes/minhas/.</t>
         </is>
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Organização</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -3533,32 +3533,32 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-001</t>
+          <t>RF-VOL-014</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Entregar notificação em tempo real</t>
+          <t>Publicar campanha de doação</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>O aviso chega sem recarregar a página.</t>
+          <t>A organização cadastra uma arrecadação de itens, como agasalhos ou alimentos, definindo como a contribuição será contada.</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>WebSocket em /ws/notificacoes/ com Django Channels sobre Daphne. Sala por usuário. Camada em Redis quando disponível, com queda para camada em memória em implantação de instância única.</t>
+          <t>Modalidade da oportunidade. A unidade é texto livre — peças de agasalho, quilos de alimento — porque qualquer lista fixa não teria a categoria da próxima campanha. Meta é opcional. Vagas e carga horária não se aplicam: campanha não limita participantes nem cumpre hora.</t>
         </is>
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -3573,32 +3573,32 @@
       </c>
       <c r="B75" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-002</t>
+          <t>RF-VOL-015</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Listar notificações</t>
+          <t>Declarar doação</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê o histórico de avisos e quantos estão por ler.</t>
+          <t>Estudante informa quanto pretende entregar à campanha.</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>GET /api/notificacoes/ e /nao-lidas/.</t>
+          <t>POST em inscrever, com quantidade declarada e descrição opcional do item. É declaração de intenção: o valor fica registrado à parte e não entra na contagem da campanha até a organização confirmar o recebimento.</t>
         </is>
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Aluno</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -3613,37 +3613,37 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-003</t>
+          <t>RF-VOL-016</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>Marcar notificação como lida</t>
+          <t>Confirmar recebimento da doação</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>Usuário marca um aviso ou todos de uma vez.</t>
+          <t>A organização registra quanto de fato recebeu, que pode divergir do que foi declarado.</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>POST /api/notificacoes/{id}/marcar-lida/ e /marcar-todas-lidas/.</t>
+          <t>POST em concluir, com a quantidade confirmada. Sem valor informado, vale o declarado. O campo é somente leitura para o estudante: se ele pudesse registrar o próprio recebimento, o total da campanha deixaria de significar algo. Emite o certificado na mesma operação.</t>
         </is>
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>CRÍTICA</t>
         </is>
       </c>
     </row>
@@ -3653,27 +3653,27 @@
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>RF-NOT-004</t>
+          <t>RF-VOL-017</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Limpar notificações</t>
+          <t>Acompanhar a arrecadação</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Usuário descarta os avisos já lidos.</t>
+          <t>A página da campanha mostra quanto já foi arrecadado e, havendo meta, o progresso em relação a ela.</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>POST /api/notificacoes/limpar/.</t>
+          <t>Soma apenas as quantidades confirmadas em participações concluídas. Sem meta declarada não há barra de progresso: a barra precisa de um denominador, e inventar um faria a campanha parecer mais adiantada do que está.</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="H77" s="9" t="inlineStr">
         <is>
-          <t>DESEJÁVEL</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3693,27 +3693,27 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>RF-NOT-005</t>
+          <t>RF-VOL-018</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Agrupar aviso por conversa</t>
+          <t>Certificar participação em campanha</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>Notificações</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>Uma conversa com muitas mensagens novas gera um aviso, e não um por mensagem.</t>
+          <t>Quem doou recebe certificado declarando a contribuição.</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>Enquanto houver aviso não lido daquela conversa, não se cria outro. Sem isso, uma discussão ativa produziria dezenas de avisos e a pessoa desligaria todos.</t>
+          <t>O texto do certificado muda com a modalidade: registra o que foi entregue e acrescenta que a organização atribui àquela participação o equivalente a um número de horas por ela definido. A formulação é deliberada — doar não é cumprir hora, e quem receber o documento precisa saber que avalia uma equivalência declarada pela entidade.</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3733,32 +3733,32 @@
       </c>
       <c r="B79" s="9" t="inlineStr">
         <is>
-          <t>RF-PRF-001</t>
+          <t>RF-VOL-019</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Visualizar perfil</t>
+          <t>Validar certificado pelo código</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Perfil</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Usuário vê seus dados, foto, curso, período e disciplinas.</t>
+          <t>Qualquer pessoa confere a autenticidade de um certificado informando o código, sem precisar de conta.</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Compõe dados de /api/auth/me/ com o andamento por disciplina.</t>
+          <t>GET /api/voluntariado/certificados/validar/{codigo}/, com acesso público (AllowAny). Devolve {valido, certificado} com dados da participação e o CPF do estudante mascarado. Permite que terceiros, como a instância que valida horas complementares, verifiquem sem depender da organização emissora.</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Visitante</t>
         </is>
       </c>
       <c r="H79" s="9" t="inlineStr">
@@ -3773,32 +3773,32 @@
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>RF-PRF-002</t>
+          <t>RF-VOL-020</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Consultar histórico de participação</t>
+          <t>Assinar o certificado em nome da organização</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
         <is>
-          <t>Perfil</t>
+          <t>Voluntariado</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>Usuário vê suas publicações, inscrições e certificados reunidos.</t>
+          <t>O certificado traz o nome, o cargo e a assinatura do responsável pela organização.</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>Agrega as consultas de cada módulo na tela de perfil.</t>
+          <t>A organização cadastra nome_responsavel, cargo_responsavel e a imagem de assinatura no próprio perfil. O serviço de emissão (voluntariado/services.py) leva esses dados ao modelo HTML do certificado.</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H80" s="8" t="inlineStr">
@@ -3813,32 +3813,32 @@
       </c>
       <c r="B81" s="9" t="inlineStr">
         <is>
-          <t>RF-COO-001</t>
+          <t>RF-PAI-001</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>Acompanhar o curso por disciplina</t>
+          <t>Painel de quem conduz a turma</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Painéis</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>A coordenação vê o movimento de cada disciplina do curso: volume de dúvidas, proporção respondida e tempo até a primeira resposta.</t>
+          <t>Professor e monitor veem, num lugar só, as dúvidas sem resposta, os pedidos de ajuda abertos e os trabalhos em andamento das suas turmas.</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>Painel que agrega por disciplina e período. Identifica disciplina com muita dúvida sem resposta, que é o sinal que o painel existe para produzir.</t>
+          <t>Composição das consultas dos módulos, restrita às disciplinas em que a pessoa leciona ou exerce monitoria. O monitor vê apenas onde é monitor.</t>
         </is>
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Professor/Monitor</t>
         </is>
       </c>
       <c r="H81" s="9" t="inlineStr">
@@ -3853,37 +3853,37 @@
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>RF-COO-002</t>
+          <t>RF-PAI-002</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Detalhar uma disciplina</t>
+          <t>Painel da organização parceira</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Painéis</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>A coordenação abre uma disciplina e vê as dúvidas mais vistas e as sem resposta.</t>
+          <t>A organização vê suas oportunidades, quantos se inscreveram e quantos concluíram.</t>
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>Consulta por disciplina, ordenada pela razão entre visualizações e respostas.</t>
+          <t>Restrito às oportunidades da própria organização. A organização não participa do fórum: publica ações, acompanha inscrições e emite certificados.</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Organização</t>
         </is>
       </c>
       <c r="H82" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3893,37 +3893,37 @@
       </c>
       <c r="B83" s="9" t="inlineStr">
         <is>
-          <t>RF-COO-003</t>
+          <t>RF-NOT-001</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>Importar a matriz curricular</t>
+          <t>Entregar notificação em tempo real</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>As disciplinas do curso entram na plataforma a partir do projeto pedagógico.</t>
+          <t>O aviso chega sem recarregar a página.</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Comando importar_matriz_ppc, que lê o ementário e cadastra código, nome, período e carga horária. A paridade do período define o semestre de oferta.</t>
+          <t>WebSocket em /ws/notificacoes/ com Django Channels sobre Daphne. Sala por usuário. Camada em Redis quando disponível, com queda para camada em memória em implantação de instância única.</t>
         </is>
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>Coordenação</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="H83" s="9" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3933,37 +3933,37 @@
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>RF-AUD-001</t>
+          <t>RF-NOT-002</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Registrar ações sensíveis</t>
+          <t>Listar notificações</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>Auditoria</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t>Ações de moderação e de gestão de vínculos ficam registradas.</t>
+          <t>Usuário vê o histórico de avisos e quantos estão por ler.</t>
         </is>
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>Modelo de registro de auditoria, com autor, ação, alvo e momento. Consulta restrita à administração.</t>
+          <t>GET /api/notificacoes/ e /nao-lidas/.</t>
         </is>
       </c>
       <c r="G84" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H84" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>ESSENCIAL</t>
         </is>
       </c>
     </row>
@@ -3973,27 +3973,27 @@
       </c>
       <c r="B85" s="9" t="inlineStr">
         <is>
-          <t>RF-SIS-001</t>
+          <t>RF-NOT-003</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>Alternar entre tema claro e escuro</t>
+          <t>Marcar notificação como lida</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Usuário escolhe o tema e a escolha permanece entre visitas.</t>
+          <t>Usuário marca um aviso ou todos de uma vez.</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>Alternância por variáveis de cor no navegador, com a preferência guardada localmente. Todas as cores da interface vêm dessas variáveis: valor fixo escrito no código produz texto ilegível num dos dois temas.</t>
+          <t>POST /api/notificacoes/{id}/marcar-lida/ e /marcar-todas-lidas/.</t>
         </is>
       </c>
       <c r="G85" s="9" t="inlineStr">
@@ -4013,37 +4013,37 @@
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>RF-SIS-002</t>
+          <t>RF-NOT-004</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Consultar a documentação da API</t>
+          <t>Limpar notificações</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Notificações</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>A especificação da API fica acessível e navegável.</t>
+          <t>Usuário descarta os avisos já lidos.</t>
         </is>
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>Esquema OpenAPI gerado por drf-spectacular a partir das views e serializadores, com interface de navegação.</t>
+          <t>POST /api/notificacoes/limpar/.</t>
         </is>
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="H86" s="8" t="inlineStr">
         <is>
-          <t>IMPORTANTE</t>
+          <t>DESEJÁVEL</t>
         </is>
       </c>
     </row>
@@ -4053,42 +4053,482 @@
       </c>
       <c r="B87" s="9" t="inlineStr">
         <is>
+          <t>RF-NOT-005</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>Agrupar aviso por conversa</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>Notificações</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>Uma conversa com muitas mensagens novas gera um aviso, e não um por mensagem.</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>Enquanto houver aviso não lido daquela conversa, não se cria outro. Sem isso, uma discussão ativa produziria dezenas de avisos e a pessoa desligaria todos.</t>
+        </is>
+      </c>
+      <c r="G87" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="H87" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>RF-PRF-001</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Visualizar perfil</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Perfil</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>Usuário vê seus dados, foto, curso, período e disciplinas.</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>Compõe dados de /api/auth/me/ com o andamento por disciplina.</t>
+        </is>
+      </c>
+      <c r="G88" s="8" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="H88" s="8" t="inlineStr">
+        <is>
+          <t>ESSENCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="9" t="inlineStr">
+        <is>
+          <t>RF-PRF-002</t>
+        </is>
+      </c>
+      <c r="C89" s="9" t="inlineStr">
+        <is>
+          <t>Consultar histórico de participação</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>Perfil</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="inlineStr">
+        <is>
+          <t>Usuário vê suas publicações, inscrições e certificados reunidos.</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="inlineStr">
+        <is>
+          <t>Agrega as consultas de cada módulo na tela de perfil.</t>
+        </is>
+      </c>
+      <c r="G89" s="9" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="H89" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>RF-COO-001</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>Acompanhar o curso por disciplina</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>A coordenação vê o movimento de cada disciplina do curso: volume de dúvidas, proporção respondida e tempo até a primeira resposta.</t>
+        </is>
+      </c>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
+          <t>Painel que agrega por disciplina e período. Identifica disciplina com muita dúvida sem resposta, que é o sinal que o painel existe para produzir.</t>
+        </is>
+      </c>
+      <c r="G90" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="H90" s="8" t="inlineStr">
+        <is>
+          <t>ESSENCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="9" t="inlineStr">
+        <is>
+          <t>RF-COO-002</t>
+        </is>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>Detalhar uma disciplina</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
+        <is>
+          <t>A coordenação abre uma disciplina e vê as dúvidas mais vistas e as sem resposta.</t>
+        </is>
+      </c>
+      <c r="F91" s="9" t="inlineStr">
+        <is>
+          <t>Consulta por disciplina, ordenada pela razão entre visualizações e respostas.</t>
+        </is>
+      </c>
+      <c r="G91" s="9" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="H91" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>RF-COO-003</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>Importar a matriz curricular</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>As disciplinas do curso entram na plataforma a partir do projeto pedagógico.</t>
+        </is>
+      </c>
+      <c r="F92" s="8" t="inlineStr">
+        <is>
+          <t>Comando importar_matriz_ppc, que lê o ementário e cadastra código, nome, período e carga horária. A paridade do período define o semestre de oferta.</t>
+        </is>
+      </c>
+      <c r="G92" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="H92" s="8" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="9" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="9" t="inlineStr">
+        <is>
+          <t>RF-AUD-001</t>
+        </is>
+      </c>
+      <c r="C93" s="9" t="inlineStr">
+        <is>
+          <t>Registrar ações sensíveis</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
+        <is>
+          <t>Ações de moderação e de gestão de vínculos ficam registradas, com autor, ação e momento.</t>
+        </is>
+      </c>
+      <c r="F93" s="9" t="inlineStr">
+        <is>
+          <t>Modelo AuditLog, com usuário, ação, objeto afetado e momento, gravado junto da ação. Os registros não são apagados. A consulta está descrita em RF-AUD-002.</t>
+        </is>
+      </c>
+      <c r="G93" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="H93" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>RF-AUD-002</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>Consultar o registro de auditoria</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>Auditoria</t>
+        </is>
+      </c>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>O usuário vê o que ele próprio executou, e a administração vê tudo, com filtros.</t>
+        </is>
+      </c>
+      <c r="F94" s="8" t="inlineStr">
+        <is>
+          <t>GET /api/auditoria/ (somente leitura). Usuário comum enxerga apenas os registros em que é o autor. Administração e superusuário enxergam todos e podem filtrar por usuário. Filtros por ação e por período (data_inicio e data_fim), com ordenação por data ou ação.</t>
+        </is>
+      </c>
+      <c r="G94" s="8" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="H94" s="8" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="9" t="inlineStr">
+        <is>
+          <t>RF-SIS-001</t>
+        </is>
+      </c>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>Alternar entre tema claro e escuro</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="inlineStr">
+        <is>
+          <t>Usuário escolhe o tema e a escolha permanece entre visitas.</t>
+        </is>
+      </c>
+      <c r="F95" s="9" t="inlineStr">
+        <is>
+          <t>Alternância por variáveis de cor no navegador, com a preferência guardada localmente. Todas as cores da interface vêm dessas variáveis: valor fixo escrito no código produz texto ilegível num dos dois temas.</t>
+        </is>
+      </c>
+      <c r="G95" s="9" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="H95" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>RF-SIS-002</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>Consultar a documentação da API</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>A especificação da API fica acessível e navegável.</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>Esquema OpenAPI gerado por drf-spectacular a partir das views e serializadores, com interface de navegação.</t>
+        </is>
+      </c>
+      <c r="G96" s="8" t="inlineStr">
+        <is>
+          <t>Desenvolvedor</t>
+        </is>
+      </c>
+      <c r="H96" s="8" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="9" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="9" t="inlineStr">
+        <is>
           <t>RF-SIS-003</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
+      <c r="C97" s="9" t="inlineStr">
         <is>
           <t>Carregar dados de demonstração</t>
         </is>
       </c>
-      <c r="D87" s="9" t="inlineStr">
+      <c r="D97" s="9" t="inlineStr">
         <is>
           <t>Sistema</t>
         </is>
       </c>
-      <c r="E87" s="9" t="inlineStr">
+      <c r="E97" s="9" t="inlineStr">
         <is>
           <t>A plataforma pode ser povoada com um semestre completo para demonstração e avaliação.</t>
         </is>
       </c>
-      <c r="F87" s="9" t="inlineStr">
+      <c r="F97" s="9" t="inlineStr">
         <is>
           <t>Comando popular_demonstracao, com semente fixa para que a mesma execução produza sempre o mesmo conjunto. Gera disciplinas com ritmos distintos de atividade, deliberadamente incluindo uma sem professor atribuído, para que o painel de coordenação tenha o que apontar.</t>
         </is>
       </c>
-      <c r="G87" s="9" t="inlineStr">
+      <c r="G97" s="9" t="inlineStr">
         <is>
           <t>Coordenação</t>
         </is>
       </c>
-      <c r="H87" s="9" t="inlineStr">
+      <c r="H97" s="9" t="inlineStr">
         <is>
           <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>RF-SIS-004</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Criar perfis de demonstração</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>Cria um usuário de cada perfil, com dados para navegar o sistema e avaliar como cada papel o enxerga.</t>
+        </is>
+      </c>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>Comando criar_perfis_demo, idempotente (rodar de novo atualiza em vez de duplicar). Contas já nascem ativas e com senhas conhecidas, então não deve ser usado em produção. Sem esses dados várias telas, como a fila de moderação e o painel de andamento, aparecem vazias.</t>
+        </is>
+      </c>
+      <c r="G98" s="8" t="inlineStr">
+        <is>
+          <t>Coordenação</t>
+        </is>
+      </c>
+      <c r="H98" s="8" t="inlineStr">
+        <is>
+          <t>DESEJÁVEL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H87"/>
+  <autoFilter ref="A1:H98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4099,7 +4539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4361,8 +4801,308 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Recuperação de senha por e-mail</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Não implementado</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>RF-AUT-002 do TCC1</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>A ativação por código cobre o primeiro acesso, mas não existe fluxo de redefinição de senha. Lacuna conhecida. A confirmar com a autora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Logout por inatividade (15 minutos)</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Não implementado</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>RF-AUT-004 do TCC1</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>A sessão expira pelo tempo dos tokens: 60 minutos de acesso e 7 dias de renovação, com rotação do token de renovação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Limite global de requisições e bloqueio de login</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Reduzido</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>RF-AUT-001 do TCC1</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Existe limite de tentativas apenas na ativação de conta por código (anti-força-bruta). Não há limitação de taxa por usuário ou IP na API. Lacuna registrada na aba Lacunas conhecidas dos não funcionais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>reCAPTCHA na inscrição e na confirmação</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Não implementado</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>RF-VOL-003 e RF-VOL-009 do TCC1</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>A integridade das inscrições é garantida por unicidade no banco, atomicidade e aprovação pela organização. A confirmar com a autora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Tópico anônimo e categorias (dúvida, discussão, anúncio)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Não implementado</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>RF-FOR-004 e RF-FOR-013 do TCC1</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>A publicação é sempre identificada e vinculada à disciplina. A confirmar com a autora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Menção a pessoas com @nome</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Não implementado</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>RF-NOT-002 do TCC1</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>As notificações cobrem resposta, mensagem, denúncia, pedido de ajuda e inscrição. Menção não foi implementada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Cifra em repouso das mensagens (AES-256)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Não implementado</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>RF-FOR-018, RF-FOR-019 e RF-FOR-020 do TCC1</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>As mensagens ficam em texto no banco. A proteção é por controle de acesso e participação na conversa (RNF-PRI-001). Lacuna registrada na aba Lacunas conhecidas dos não funcionais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Chat aluno-professor com sub-chats por dúvida</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Substituído</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>RF-FOR-019 do TCC1</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Substituído pelo encaminhamento seletivo do pedido de ajuda (RF-COL-011 a RF-COL-013), que preserva a privacidade da conversa do grupo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Chat monitor-professor</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Incorporado</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>RF-FOR-018 do TCC1</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Implementado como canal da monitoria por disciplina, com arquivamento ao fim da monitoria (RF-COL-019 e RF-COL-020).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Grupos de trabalho com período e encerramento automático</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Reformulado</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>RF-FOR-020 e RF-FOR-021 do TCC1</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Passou a ser o módulo de trabalhos em grupo, com prazo de entrega, formação por escolha ou sorteio e conversa por grupo (RF-COL-001 a RF-COL-010).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Upload de vídeo e geocodificação das oportunidades</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Reduzido</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>RF-VOL-002 e RF-VOL-005 do TCC1</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>A oportunidade tem imagem de capa e local em texto livre. Não há vídeo nem coordenadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Busca unificada de usuários, tópicos e oportunidades</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Reduzido</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>RF-PRF-006 do TCC1</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>A busca atende ao fórum (RF-FOR-019). A localização de pessoas é restrita a quem gere papéis (RF-AUT-009).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:E22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Corrige o ator de RF-COL-001, 003 e 004 para Professor
O código só deixa o professor da disciplina propor o trabalho, criar os
grupos e sortear a composição. A planilha ainda listava Professor/Monitor
nesses três requisitos. As planilhas foram regeneradas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
+++ b/docs/Requisitos_Funcionais_Plataforma_UNIFEI.xlsx
@@ -2153,12 +2153,12 @@
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/. Exige que a pessoa lecione a disciplina — a coordenação não passa nesta verificação, porque supervisionar não é participar da turma.</t>
+          <t>POST /api/colaboracao/trabalhos/. Exige que a pessoa lecione a disciplina — a coordenação não passa nesta verificação, porque supervisionar não é participar da turma. O monitor também não passa: ele costuma ser aluno de período próximo, e criar a atividade pela qual os colegas serão avaliados inverteria a relação da monitoria.</t>
         </is>
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="H39" s="9" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/{id}/criar-grupos/. Cria a conversa privada de cada grupo junto.</t>
+          <t>POST /api/colaboracao/trabalhos/{id}/criar-grupos/. Cria a conversa privada de cada grupo junto. Restrito ao professor da disciplina.</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="H41" s="9" t="inlineStr">
@@ -2273,12 +2273,12 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>POST /api/colaboracao/trabalhos/{id}/sortear/. Respeita o tamanho máximo e sincroniza os participantes das conversas.</t>
+          <t>POST /api/colaboracao/trabalhos/{id}/sortear/. Respeita o tamanho máximo e sincroniza os participantes das conversas. Restrito ao professor da disciplina.</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>Professor/Monitor</t>
+          <t>Professor</t>
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr">

</xml_diff>